<commit_message>
Cabeça do pilar: dois aparelhos com junta central
Volta x,ap para a,cab/2 − h,pil/2 − F,ap (borda externa do aparelho além da
face do pilar), pois a0 é a soma de dois aparelhos com junta 2·(c+f) no
centro. O desenho passa a mostrar os dois aparelhos separados pela junta.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q3cH5Ra5NbDLqkpmKm8CnH
</commit_message>
<xml_diff>
--- a/34 - Bloco Parcialmente carregado.xlsx
+++ b/34 - Bloco Parcialmente carregado.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Cabeça do pilar" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Cabeça do pilar'!$K$1:$T$321</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Cabeça do pilar'!$K$1:$T$327</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1" iterateCount="1000"/>
 </workbook>
@@ -462,7 +462,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$L$219:$L$223</c:f>
+              <c:f>'Cabeça do pilar'!$L$219:$L$229</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
@@ -486,7 +486,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$M$219:$M$223</c:f>
+              <c:f>'Cabeça do pilar'!$M$219:$M$229</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
@@ -520,7 +520,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Cabeça do pilar'!$O$224</c:f>
+              <c:f>'Cabeça do pilar'!$O$230</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -542,7 +542,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$L$224:$L$227</c:f>
+              <c:f>'Cabeça do pilar'!$L$230:$L$233</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
@@ -563,7 +563,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$M$224:$M$227</c:f>
+              <c:f>'Cabeça do pilar'!$M$230:$M$233</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
@@ -594,7 +594,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Cabeça do pilar'!$O$228</c:f>
+              <c:f>'Cabeça do pilar'!$O$234</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -616,7 +616,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$L$228:$L$257</c:f>
+              <c:f>'Cabeça do pilar'!$L$234:$L$263</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="30"/>
@@ -685,7 +685,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$M$228:$M$257</c:f>
+              <c:f>'Cabeça do pilar'!$M$234:$M$263</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="30"/>
@@ -764,7 +764,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Cabeça do pilar'!$O$258</c:f>
+              <c:f>'Cabeça do pilar'!$O$264</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -787,7 +787,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$L$258:$L$317</c:f>
+              <c:f>'Cabeça do pilar'!$L$264:$L$323</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="60"/>
@@ -916,7 +916,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$M$258:$M$317</c:f>
+              <c:f>'Cabeça do pilar'!$M$264:$M$323</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="60"/>
@@ -1055,7 +1055,7 @@
           <c:order val="5"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Cabeça do pilar'!$O$318</c:f>
+              <c:f>'Cabeça do pilar'!$O$324</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1078,7 +1078,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$L$318:$L$319</c:f>
+              <c:f>'Cabeça do pilar'!$L$324:$L$325</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1093,7 +1093,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$M$318:$M$319</c:f>
+              <c:f>'Cabeça do pilar'!$M$324:$M$325</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1118,7 +1118,7 @@
           <c:order val="6"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Cabeça do pilar'!$O$320</c:f>
+              <c:f>'Cabeça do pilar'!$O$326</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1137,7 +1137,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$L$320:$L$321</c:f>
+              <c:f>'Cabeça do pilar'!$L$326:$L$327</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1152,7 +1152,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$M$320:$M$321</c:f>
+              <c:f>'Cabeça do pilar'!$M$326:$M$327</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1803,7 +1803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T321"/>
+  <dimension ref="A1:T327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.7109375" customWidth="1" style="15" min="10" max="10"/>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="O43" s="3" t="inlineStr">
         <is>
-          <t>Comprimento do aparelho de apoio (direção de a,cab).</t>
+          <t>Soma dos 2 aparelhos (uma viga de cada lado). No centro fica a junta vazia entre as vigas: 2·(c + f).</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2883,7 @@
         </is>
       </c>
       <c r="L65" s="23">
-        <f>(L43-L32)/2</f>
+        <f>L37/2-L32/2-L42</f>
         <v/>
       </c>
       <c r="M65" s="2" t="inlineStr">
@@ -2893,7 +2893,7 @@
       </c>
       <c r="O65" s="3" t="inlineStr">
         <is>
-          <t>(a0 − h,pil)/2: parte do aparelho fora da face do pilar, de cada lado. ≤ 0 → todo sobre o pilar.</t>
+          <t>a,cab/2 − h,pil/2 − F,ap: quanto a borda externa do aparelho passa da face do pilar. ≤ 0 → todo sobre o pilar.</t>
         </is>
       </c>
     </row>
@@ -3836,7 +3836,7 @@
         </is>
       </c>
       <c r="L124" s="6">
-        <f>MAX(0,L65)</f>
+        <f>MAX(0,MIN(L65,L43/2))</f>
         <v/>
       </c>
       <c r="M124" s="2" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="O124" s="3" t="inlineStr">
         <is>
-          <t>Parte do aparelho fora da face do pilar, de cada lado: (a0 − h,pil)/2 ≥ 0 (item 1.7).</t>
+          <t>Parte do aparelho fora da face do pilar, de cada lado (item 1.7; limitada a a0/2).</t>
         </is>
       </c>
     </row>
@@ -4710,7 +4710,7 @@
         </is>
       </c>
       <c r="L219" s="6">
-        <f>-L43/2</f>
+        <f>-(L37/2-L42)</f>
         <v/>
       </c>
       <c r="M219" s="6">
@@ -4718,13 +4718,13 @@
         <v/>
       </c>
       <c r="O219" s="3">
-        <f>"Aparelho de apoio "&amp;L43&amp;" × "&amp;L44&amp;" cm"</f>
+        <f>"Aparelhos 2 × "&amp;L43/2&amp;" × "&amp;L44&amp;" cm (junta "&amp;2*(L37/2-L42-L43/2)&amp;" cm)"</f>
         <v/>
       </c>
     </row>
     <row r="220">
       <c r="L220" s="6">
-        <f>L43/2</f>
+        <f>-(L37/2-L42-L43/2)</f>
         <v/>
       </c>
       <c r="M220" s="6">
@@ -4734,7 +4734,7 @@
     </row>
     <row r="221">
       <c r="L221" s="6">
-        <f>L43/2</f>
+        <f>-(L37/2-L42-L43/2)</f>
         <v/>
       </c>
       <c r="M221" s="6">
@@ -4744,7 +4744,7 @@
     </row>
     <row r="222">
       <c r="L222" s="6">
-        <f>-L43/2</f>
+        <f>-(L37/2-L42)</f>
         <v/>
       </c>
       <c r="M222" s="6">
@@ -4754,7 +4754,7 @@
     </row>
     <row r="223">
       <c r="L223" s="6">
-        <f>-L43/2</f>
+        <f>-(L37/2-L42)</f>
         <v/>
       </c>
       <c r="M223" s="6">
@@ -4763,752 +4763,804 @@
       </c>
     </row>
     <row r="224">
-      <c r="K224" s="1" t="inlineStr">
-        <is>
-          <t>Tirante</t>
-        </is>
-      </c>
-      <c r="L224" s="6">
-        <f>-(L37/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M224" s="6">
-        <f>(-(L35+L107/20))-(L107)</f>
-        <v/>
-      </c>
-      <c r="O224" s="3">
-        <f>"Tirante "&amp;L108&amp;" Ø"&amp;L107&amp;IF(L68="Bloco"," (bloco)"," (consolo)")</f>
-        <v/>
-      </c>
+      <c r="L224" s="6" t="n"/>
+      <c r="M224" s="6" t="n"/>
     </row>
     <row r="225">
       <c r="L225" s="6">
-        <f>-(L37/2-L35)</f>
+        <f>(L37/2-L42-L43/2)</f>
         <v/>
       </c>
       <c r="M225" s="6">
-        <f>(-(L35+L107/20))</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
     <row r="226">
       <c r="L226" s="6">
-        <f>(L37/2-L35)</f>
+        <f>L37/2-L42</f>
         <v/>
       </c>
       <c r="M226" s="6">
-        <f>(-(L35+L107/20))</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
     <row r="227">
       <c r="L227" s="6">
-        <f>(L37/2-L35)</f>
+        <f>L37/2-L42</f>
         <v/>
       </c>
       <c r="M227" s="6">
-        <f>(-(L35+L107/20))-(L107)</f>
+        <f>MAX(L45,2)</f>
         <v/>
       </c>
     </row>
     <row r="228">
-      <c r="K228" s="1" t="inlineStr">
-        <is>
-          <t>Costura</t>
-        </is>
-      </c>
       <c r="L228" s="6">
-        <f>IF(L141=0,L318,-(IF((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>(L37/2-L42-L43/2)</f>
         <v/>
       </c>
       <c r="M228" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))</f>
-        <v/>
-      </c>
-      <c r="O228" s="3">
-        <f>IF(L141=0,"Costura – não se aplica (bloco)","Costura "&amp;L141&amp;" Ø"&amp;L139&amp;" c/"&amp;L142)</f>
+        <f>MAX(L45,2)</f>
         <v/>
       </c>
     </row>
     <row r="229">
       <c r="L229" s="6">
-        <f>IF(L141=0,L318,(IF((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>(L37/2-L42-L43/2)</f>
         <v/>
       </c>
       <c r="M229" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="230"/>
+        <f>0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="230">
+      <c r="K230" s="1" t="inlineStr">
+        <is>
+          <t>Tirante</t>
+        </is>
+      </c>
+      <c r="L230" s="6">
+        <f>-(L37/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M230" s="6">
+        <f>(-(L35+L107/20))-(L107)</f>
+        <v/>
+      </c>
+      <c r="O230" s="3">
+        <f>"Tirante "&amp;L108&amp;" Ø"&amp;L107&amp;IF(L68="Bloco"," (bloco)"," (consolo)")</f>
+        <v/>
+      </c>
+    </row>
     <row r="231">
       <c r="L231" s="6">
-        <f>IF(L141=0,L318,-(IF((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>-(L37/2-L35)</f>
         <v/>
       </c>
       <c r="M231" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))</f>
+        <f>(-(L35+L107/20))</f>
         <v/>
       </c>
     </row>
     <row r="232">
       <c r="L232" s="6">
-        <f>IF(L141=0,L318,(IF((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>(L37/2-L35)</f>
         <v/>
       </c>
       <c r="M232" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="233"/>
+        <f>(-(L35+L107/20))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="233">
+      <c r="L233" s="6">
+        <f>(L37/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M233" s="6">
+        <f>(-(L35+L107/20))-(L107)</f>
+        <v/>
+      </c>
+    </row>
     <row r="234">
+      <c r="K234" s="1" t="inlineStr">
+        <is>
+          <t>Costura</t>
+        </is>
+      </c>
       <c r="L234" s="6">
-        <f>IF(L141=0,L318,-(IF((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M234" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))</f>
+        <v/>
+      </c>
+      <c r="O234" s="3">
+        <f>IF(L141=0,"Costura – não se aplica (bloco)","Costura "&amp;L141&amp;" Ø"&amp;L139&amp;" c/"&amp;L142)</f>
         <v/>
       </c>
     </row>
     <row r="235">
       <c r="L235" s="6">
-        <f>IF(L141=0,L318,(IF((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M235" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="236"/>
     <row r="237">
       <c r="L237" s="6">
-        <f>IF(L141=0,L318,-(IF((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M237" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="238">
       <c r="L238" s="6">
-        <f>IF(L141=0,L318,(IF((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M238" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="239"/>
     <row r="240">
       <c r="L240" s="6">
-        <f>IF(L141=0,L318,-(IF((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M240" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="241">
       <c r="L241" s="6">
-        <f>IF(L141=0,L318,(IF((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M241" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="242"/>
     <row r="243">
       <c r="L243" s="6">
-        <f>IF(L141=0,L318,-(IF((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M243" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="244">
       <c r="L244" s="6">
-        <f>IF(L141=0,L318,(IF((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M244" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="245"/>
     <row r="246">
       <c r="L246" s="6">
-        <f>IF(L141=0,L318,-(IF((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M246" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="247">
       <c r="L247" s="6">
-        <f>IF(L141=0,L318,(IF((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M247" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="248"/>
     <row r="249">
       <c r="L249" s="6">
-        <f>IF(L141=0,L318,-(IF((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M249" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="250">
       <c r="L250" s="6">
-        <f>IF(L141=0,L318,(IF((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M250" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="251"/>
     <row r="252">
       <c r="L252" s="6">
-        <f>IF(L141=0,L318,-(IF((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M252" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="253">
       <c r="L253" s="6">
-        <f>IF(L141=0,L318,(IF((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M253" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="254"/>
     <row r="255">
       <c r="L255" s="6">
-        <f>IF(L141=0,L318,-(IF((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M255" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="256">
       <c r="L256" s="6">
-        <f>IF(L141=0,L318,(IF((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M256" s="6">
-        <f>IF(L141=0,M318,((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="257"/>
     <row r="258">
-      <c r="K258" s="1" t="inlineStr">
-        <is>
-          <t>Cintas</t>
-        </is>
-      </c>
       <c r="L258" s="6">
-        <f>-(IF((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M258" s="6">
-        <f>(-(IF(1&lt;=L96,1,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-      <c r="O258" s="3">
-        <f>"Cintas "&amp;L96&amp;" Ø"&amp;L94&amp;" c/"&amp;L97</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="259">
       <c r="L259" s="6">
-        <f>(IF((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M259" s="6">
-        <f>(-(IF(1&lt;=L96,1,1)-0.5)*L97)</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="260"/>
     <row r="261">
       <c r="L261" s="6">
-        <f>-(IF((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M261" s="6">
-        <f>(-(IF(2&lt;=L96,2,1)-0.5)*L97)</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="262">
       <c r="L262" s="6">
-        <f>(IF((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M262" s="6">
-        <f>(-(IF(2&lt;=L96,2,1)-0.5)*L97)</f>
+        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))</f>
         <v/>
       </c>
     </row>
     <row r="263"/>
     <row r="264">
+      <c r="K264" s="1" t="inlineStr">
+        <is>
+          <t>Cintas</t>
+        </is>
+      </c>
       <c r="L264" s="6">
-        <f>-(IF((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M264" s="6">
-        <f>(-(IF(3&lt;=L96,3,1)-0.5)*L97)</f>
+        <f>(-(IF(1&lt;=L96,1,1)-0.5)*L97)</f>
+        <v/>
+      </c>
+      <c r="O264" s="3">
+        <f>"Cintas "&amp;L96&amp;" Ø"&amp;L94&amp;" c/"&amp;L97</f>
         <v/>
       </c>
     </row>
     <row r="265">
       <c r="L265" s="6">
-        <f>(IF((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M265" s="6">
-        <f>(-(IF(3&lt;=L96,3,1)-0.5)*L97)</f>
+        <f>(-(IF(1&lt;=L96,1,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="266"/>
     <row r="267">
       <c r="L267" s="6">
-        <f>-(IF((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M267" s="6">
-        <f>(-(IF(4&lt;=L96,4,1)-0.5)*L97)</f>
+        <f>(-(IF(2&lt;=L96,2,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="268">
       <c r="L268" s="6">
-        <f>(IF((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M268" s="6">
-        <f>(-(IF(4&lt;=L96,4,1)-0.5)*L97)</f>
+        <f>(-(IF(2&lt;=L96,2,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="269"/>
     <row r="270">
       <c r="L270" s="6">
-        <f>-(IF((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M270" s="6">
-        <f>(-(IF(5&lt;=L96,5,1)-0.5)*L97)</f>
+        <f>(-(IF(3&lt;=L96,3,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="271">
       <c r="L271" s="6">
-        <f>(IF((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M271" s="6">
-        <f>(-(IF(5&lt;=L96,5,1)-0.5)*L97)</f>
+        <f>(-(IF(3&lt;=L96,3,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="272"/>
     <row r="273">
       <c r="L273" s="6">
-        <f>-(IF((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M273" s="6">
-        <f>(-(IF(6&lt;=L96,6,1)-0.5)*L97)</f>
+        <f>(-(IF(4&lt;=L96,4,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="274">
       <c r="L274" s="6">
-        <f>(IF((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M274" s="6">
-        <f>(-(IF(6&lt;=L96,6,1)-0.5)*L97)</f>
+        <f>(-(IF(4&lt;=L96,4,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="275"/>
     <row r="276">
       <c r="L276" s="6">
-        <f>-(IF((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M276" s="6">
-        <f>(-(IF(7&lt;=L96,7,1)-0.5)*L97)</f>
+        <f>(-(IF(5&lt;=L96,5,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="277">
       <c r="L277" s="6">
-        <f>(IF((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M277" s="6">
-        <f>(-(IF(7&lt;=L96,7,1)-0.5)*L97)</f>
+        <f>(-(IF(5&lt;=L96,5,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="278"/>
     <row r="279">
       <c r="L279" s="6">
-        <f>-(IF((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M279" s="6">
-        <f>(-(IF(8&lt;=L96,8,1)-0.5)*L97)</f>
+        <f>(-(IF(6&lt;=L96,6,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="280">
       <c r="L280" s="6">
-        <f>(IF((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M280" s="6">
-        <f>(-(IF(8&lt;=L96,8,1)-0.5)*L97)</f>
+        <f>(-(IF(6&lt;=L96,6,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="281"/>
     <row r="282">
       <c r="L282" s="6">
-        <f>-(IF((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M282" s="6">
-        <f>(-(IF(9&lt;=L96,9,1)-0.5)*L97)</f>
+        <f>(-(IF(7&lt;=L96,7,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="283">
       <c r="L283" s="6">
-        <f>(IF((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M283" s="6">
-        <f>(-(IF(9&lt;=L96,9,1)-0.5)*L97)</f>
+        <f>(-(IF(7&lt;=L96,7,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="284"/>
     <row r="285">
       <c r="L285" s="6">
-        <f>-(IF((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M285" s="6">
-        <f>(-(IF(10&lt;=L96,10,1)-0.5)*L97)</f>
+        <f>(-(IF(8&lt;=L96,8,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="286">
       <c r="L286" s="6">
-        <f>(IF((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M286" s="6">
-        <f>(-(IF(10&lt;=L96,10,1)-0.5)*L97)</f>
+        <f>(-(IF(8&lt;=L96,8,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="287"/>
     <row r="288">
       <c r="L288" s="6">
-        <f>-(IF((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M288" s="6">
-        <f>(-(IF(11&lt;=L96,11,1)-0.5)*L97)</f>
+        <f>(-(IF(9&lt;=L96,9,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="289">
       <c r="L289" s="6">
-        <f>(IF((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M289" s="6">
-        <f>(-(IF(11&lt;=L96,11,1)-0.5)*L97)</f>
+        <f>(-(IF(9&lt;=L96,9,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="290"/>
     <row r="291">
       <c r="L291" s="6">
-        <f>-(IF((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M291" s="6">
-        <f>(-(IF(12&lt;=L96,12,1)-0.5)*L97)</f>
+        <f>(-(IF(10&lt;=L96,10,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="292">
       <c r="L292" s="6">
-        <f>(IF((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M292" s="6">
-        <f>(-(IF(12&lt;=L96,12,1)-0.5)*L97)</f>
+        <f>(-(IF(10&lt;=L96,10,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="293"/>
     <row r="294">
       <c r="L294" s="6">
-        <f>-(IF((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M294" s="6">
-        <f>(-(IF(13&lt;=L96,13,1)-0.5)*L97)</f>
+        <f>(-(IF(11&lt;=L96,11,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="295">
       <c r="L295" s="6">
-        <f>(IF((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M295" s="6">
-        <f>(-(IF(13&lt;=L96,13,1)-0.5)*L97)</f>
+        <f>(-(IF(11&lt;=L96,11,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="296"/>
     <row r="297">
       <c r="L297" s="6">
-        <f>-(IF((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M297" s="6">
-        <f>(-(IF(14&lt;=L96,14,1)-0.5)*L97)</f>
+        <f>(-(IF(12&lt;=L96,12,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="298">
       <c r="L298" s="6">
-        <f>(IF((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M298" s="6">
-        <f>(-(IF(14&lt;=L96,14,1)-0.5)*L97)</f>
+        <f>(-(IF(12&lt;=L96,12,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="299"/>
     <row r="300">
       <c r="L300" s="6">
-        <f>-(IF((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M300" s="6">
-        <f>(-(IF(15&lt;=L96,15,1)-0.5)*L97)</f>
+        <f>(-(IF(13&lt;=L96,13,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="301">
       <c r="L301" s="6">
-        <f>(IF((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M301" s="6">
-        <f>(-(IF(15&lt;=L96,15,1)-0.5)*L97)</f>
+        <f>(-(IF(13&lt;=L96,13,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="302"/>
     <row r="303">
       <c r="L303" s="6">
-        <f>-(IF((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M303" s="6">
-        <f>(-(IF(16&lt;=L96,16,1)-0.5)*L97)</f>
+        <f>(-(IF(14&lt;=L96,14,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="304">
       <c r="L304" s="6">
-        <f>(IF((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M304" s="6">
-        <f>(-(IF(16&lt;=L96,16,1)-0.5)*L97)</f>
+        <f>(-(IF(14&lt;=L96,14,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="305"/>
     <row r="306">
       <c r="L306" s="6">
-        <f>-(IF((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M306" s="6">
-        <f>(-(IF(17&lt;=L96,17,1)-0.5)*L97)</f>
+        <f>(-(IF(15&lt;=L96,15,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="307">
       <c r="L307" s="6">
-        <f>(IF((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M307" s="6">
-        <f>(-(IF(17&lt;=L96,17,1)-0.5)*L97)</f>
+        <f>(-(IF(15&lt;=L96,15,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="309">
       <c r="L309" s="6">
-        <f>-(IF((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M309" s="6">
-        <f>(-(IF(18&lt;=L96,18,1)-0.5)*L97)</f>
+        <f>(-(IF(16&lt;=L96,16,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="310">
       <c r="L310" s="6">
-        <f>(IF((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M310" s="6">
-        <f>(-(IF(18&lt;=L96,18,1)-0.5)*L97)</f>
+        <f>(-(IF(16&lt;=L96,16,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="312">
       <c r="L312" s="6">
-        <f>-(IF((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M312" s="6">
-        <f>(-(IF(19&lt;=L96,19,1)-0.5)*L97)</f>
+        <f>(-(IF(17&lt;=L96,17,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="313">
       <c r="L313" s="6">
-        <f>(IF((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M313" s="6">
-        <f>(-(IF(19&lt;=L96,19,1)-0.5)*L97)</f>
+        <f>(-(IF(17&lt;=L96,17,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="315">
       <c r="L315" s="6">
-        <f>-(IF((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M315" s="6">
-        <f>(-(IF(20&lt;=L96,20,1)-0.5)*L97)</f>
+        <f>(-(IF(18&lt;=L96,18,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="316">
       <c r="L316" s="6">
-        <f>(IF((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>(IF((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M316" s="6">
-        <f>(-(IF(20&lt;=L96,20,1)-0.5)*L97)</f>
+        <f>(-(IF(18&lt;=L96,18,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="318">
-      <c r="K318" s="1" t="inlineStr">
-        <is>
-          <t>Eixo</t>
-        </is>
-      </c>
       <c r="L318" s="6">
-        <f>0</f>
+        <f>-(IF((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M318" s="6">
-        <f>MAX(L45,2)+8</f>
-        <v/>
-      </c>
-      <c r="O318" s="3">
-        <f>"Eixo do pilar"</f>
+        <f>(-(IF(19&lt;=L96,19,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="319">
       <c r="L319" s="6">
-        <f>0</f>
+        <f>(IF((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M319" s="6">
-        <f>-(L120+MAX(40,L93-L120+10))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="320">
-      <c r="K320" s="1" t="inlineStr">
-        <is>
-          <t>Moldura</t>
-        </is>
-      </c>
-      <c r="L320" s="6">
-        <f>-MAX(L37+30,(L120+MAX(40,L93-L120+10))+25)/2</f>
-        <v/>
-      </c>
-      <c r="M320" s="6">
-        <f>15</f>
-        <v/>
-      </c>
-      <c r="O320" s="3">
-        <f>"(moldura – mantém a escala)"</f>
+        <f>(-(IF(19&lt;=L96,19,1)-0.5)*L97)</f>
         <v/>
       </c>
     </row>
     <row r="321">
       <c r="L321" s="6">
+        <f>-(IF((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M321" s="6">
+        <f>(-(IF(20&lt;=L96,20,1)-0.5)*L97)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="322">
+      <c r="L322" s="6">
+        <f>(IF((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M322" s="6">
+        <f>(-(IF(20&lt;=L96,20,1)-0.5)*L97)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="324">
+      <c r="K324" s="1" t="inlineStr">
+        <is>
+          <t>Eixo</t>
+        </is>
+      </c>
+      <c r="L324" s="6">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="M324" s="6">
+        <f>MAX(L45,2)+8</f>
+        <v/>
+      </c>
+      <c r="O324" s="3">
+        <f>"Eixo do pilar"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="325">
+      <c r="L325" s="6">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="M325" s="6">
+        <f>-(L120+MAX(40,L93-L120+10))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="326">
+      <c r="K326" s="1" t="inlineStr">
+        <is>
+          <t>Moldura</t>
+        </is>
+      </c>
+      <c r="L326" s="6">
+        <f>-MAX(L37+30,(L120+MAX(40,L93-L120+10))+25)/2</f>
+        <v/>
+      </c>
+      <c r="M326" s="6">
+        <f>15</f>
+        <v/>
+      </c>
+      <c r="O326" s="3">
+        <f>"(moldura – mantém a escala)"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="327">
+      <c r="L327" s="6">
         <f>MAX(L37+30,(L120+MAX(40,L93-L120+10))+25)/2</f>
         <v/>
       </c>
-      <c r="M321" s="6">
+      <c r="M327" s="6">
         <f>15-MAX(L37+30,(L120+MAX(40,L93-L120+10))+25)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Aparelho de apoio: furos por aparelho (2 aparelhos × n furos)
Adiciona a entrada n,furos (padrão 2) e Ø,furo = 4 cm; A,ap desconta
2 × n,furos furos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q3cH5Ra5NbDLqkpmKm8CnH
</commit_message>
<xml_diff>
--- a/34 - Bloco Parcialmente carregado.xlsx
+++ b/34 - Bloco Parcialmente carregado.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Cabeça do pilar" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Cabeça do pilar'!$K$1:$T$327</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Cabeça do pilar'!$K$1:$T$328</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1" iterateCount="1000"/>
 </workbook>
@@ -342,7 +342,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Cabeça do pilar'!$O$211</c:f>
+              <c:f>'Cabeça do pilar'!$O$212</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -364,7 +364,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$L$211:$L$218</c:f>
+              <c:f>'Cabeça do pilar'!$L$212:$L$219</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="8"/>
@@ -397,7 +397,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$M$211:$M$218</c:f>
+              <c:f>'Cabeça do pilar'!$M$212:$M$219</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="8"/>
@@ -440,7 +440,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Cabeça do pilar'!$O$219</c:f>
+              <c:f>'Cabeça do pilar'!$O$220</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -462,7 +462,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$L$219:$L$229</c:f>
+              <c:f>'Cabeça do pilar'!$L$220:$L$230</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
@@ -486,7 +486,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$M$219:$M$229</c:f>
+              <c:f>'Cabeça do pilar'!$M$220:$M$230</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
@@ -520,7 +520,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Cabeça do pilar'!$O$230</c:f>
+              <c:f>'Cabeça do pilar'!$O$231</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -542,7 +542,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$L$230:$L$233</c:f>
+              <c:f>'Cabeça do pilar'!$L$231:$L$234</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
@@ -563,7 +563,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$M$230:$M$233</c:f>
+              <c:f>'Cabeça do pilar'!$M$231:$M$234</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
@@ -594,7 +594,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Cabeça do pilar'!$O$234</c:f>
+              <c:f>'Cabeça do pilar'!$O$235</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -616,7 +616,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$L$234:$L$263</c:f>
+              <c:f>'Cabeça do pilar'!$L$235:$L$264</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="30"/>
@@ -685,7 +685,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$M$234:$M$263</c:f>
+              <c:f>'Cabeça do pilar'!$M$235:$M$264</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="30"/>
@@ -764,7 +764,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Cabeça do pilar'!$O$264</c:f>
+              <c:f>'Cabeça do pilar'!$O$265</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -787,7 +787,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$L$264:$L$323</c:f>
+              <c:f>'Cabeça do pilar'!$L$265:$L$324</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="60"/>
@@ -916,7 +916,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$M$264:$M$323</c:f>
+              <c:f>'Cabeça do pilar'!$M$265:$M$324</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="60"/>
@@ -1055,7 +1055,7 @@
           <c:order val="5"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Cabeça do pilar'!$O$324</c:f>
+              <c:f>'Cabeça do pilar'!$O$325</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1078,7 +1078,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$L$324:$L$325</c:f>
+              <c:f>'Cabeça do pilar'!$L$325:$L$326</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1093,7 +1093,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$M$324:$M$325</c:f>
+              <c:f>'Cabeça do pilar'!$M$325:$M$326</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1118,7 +1118,7 @@
           <c:order val="6"/>
           <c:tx>
             <c:strRef>
-              <c:f>'Cabeça do pilar'!$O$326</c:f>
+              <c:f>'Cabeça do pilar'!$O$327</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1137,7 +1137,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$L$326:$L$327</c:f>
+              <c:f>'Cabeça do pilar'!$L$327:$L$328</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1152,7 +1152,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Cabeça do pilar'!$M$326:$M$327</c:f>
+              <c:f>'Cabeça do pilar'!$M$327:$M$328</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="2"/>
@@ -1291,7 +1291,7 @@
     <xdr:from>
       <xdr:col>21</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>121</xdr:row>
+      <xdr:row>122</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1809750" cy="4876800"/>
@@ -1330,7 +1330,7 @@
     <xdr:from>
       <xdr:col>21</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>72</xdr:row>
+      <xdr:row>73</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="4953000" cy="3714750"/>
@@ -1369,7 +1369,7 @@
     <xdr:from>
       <xdr:col>21</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>97</xdr:row>
+      <xdr:row>98</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="4000500" cy="2943225"/>
@@ -1408,7 +1408,7 @@
     <xdr:from>
       <xdr:col>21</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>114</xdr:row>
+      <xdr:row>115</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1047750" cy="952500"/>
@@ -1447,13 +1447,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>165</xdr:row>
+      <xdr:row>166</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>209</xdr:row>
+      <xdr:row>210</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -1803,7 +1803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T327"/>
+  <dimension ref="A1:T328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.7109375" customWidth="1" style="15" min="10" max="10"/>
@@ -1890,12 +1890,12 @@
         </is>
       </c>
       <c r="L7" s="18">
-        <f>L68</f>
+        <f>L69</f>
         <v/>
       </c>
       <c r="M7" s="20" t="n"/>
       <c r="N7" s="5">
-        <f>N68</f>
+        <f>N69</f>
         <v/>
       </c>
       <c r="O7" s="3" t="inlineStr">
@@ -1911,7 +1911,7 @@
         </is>
       </c>
       <c r="L8" s="21">
-        <f>K69</f>
+        <f>K70</f>
         <v/>
       </c>
     </row>
@@ -1922,12 +1922,12 @@
         </is>
       </c>
       <c r="L9" s="18">
-        <f>L79</f>
+        <f>L80</f>
         <v/>
       </c>
       <c r="M9" s="20" t="n"/>
       <c r="N9" s="5">
-        <f>N79</f>
+        <f>N80</f>
         <v/>
       </c>
       <c r="O9" s="3" t="inlineStr">
@@ -1943,12 +1943,12 @@
         </is>
       </c>
       <c r="L10" s="18">
-        <f>L96&amp;" Ø"&amp;L94&amp;" c/"&amp;L97&amp;" ("&amp;L95&amp;" ramos)"</f>
+        <f>L97&amp;" Ø"&amp;L95&amp;" c/"&amp;L98&amp;" ("&amp;L96&amp;" ramos)"</f>
         <v/>
       </c>
       <c r="M10" s="20" t="n"/>
       <c r="N10" s="5">
-        <f>N96</f>
+        <f>N97</f>
         <v/>
       </c>
       <c r="O10" s="3" t="inlineStr">
@@ -1964,12 +1964,12 @@
         </is>
       </c>
       <c r="L11" s="18">
-        <f>L108&amp;" Ø"&amp;L107</f>
+        <f>L109&amp;" Ø"&amp;L108</f>
         <v/>
       </c>
       <c r="M11" s="20" t="n"/>
       <c r="N11" s="5">
-        <f>N108</f>
+        <f>N109</f>
         <v/>
       </c>
       <c r="O11" s="3" t="inlineStr">
@@ -1985,12 +1985,12 @@
         </is>
       </c>
       <c r="L12" s="18">
-        <f>L112&amp;" Ø"&amp;L111</f>
+        <f>L113&amp;" Ø"&amp;L112</f>
         <v/>
       </c>
       <c r="M12" s="20" t="n"/>
       <c r="N12" s="5">
-        <f>N112</f>
+        <f>N113</f>
         <v/>
       </c>
       <c r="O12" s="3" t="inlineStr">
@@ -2006,12 +2006,12 @@
         </is>
       </c>
       <c r="L13" s="18">
-        <f>L129</f>
+        <f>L130</f>
         <v/>
       </c>
       <c r="M13" s="20" t="n"/>
       <c r="N13" s="5">
-        <f>N121</f>
+        <f>N122</f>
         <v/>
       </c>
       <c r="O13" s="3" t="inlineStr">
@@ -2027,12 +2027,12 @@
         </is>
       </c>
       <c r="L14" s="18">
-        <f>IF(L141=0,"Não se aplica (bloco)",L141&amp;" Ø"&amp;L139&amp;" c/"&amp;L142&amp;" ("&amp;L140&amp;" ramos)")</f>
+        <f>IF(L142=0,"Não se aplica (bloco)",L142&amp;" Ø"&amp;L140&amp;" c/"&amp;L143&amp;" ("&amp;L141&amp;" ramos)")</f>
         <v/>
       </c>
       <c r="M14" s="20" t="n"/>
       <c r="N14" s="5">
-        <f>N141</f>
+        <f>N142</f>
         <v/>
       </c>
       <c r="O14" s="3" t="inlineStr">
@@ -2048,12 +2048,12 @@
         </is>
       </c>
       <c r="L15" s="18">
-        <f>L144</f>
+        <f>L145</f>
         <v/>
       </c>
       <c r="M15" s="20" t="n"/>
       <c r="N15" s="5">
-        <f>N145</f>
+        <f>N146</f>
         <v/>
       </c>
       <c r="O15" s="3" t="inlineStr">
@@ -2069,12 +2069,12 @@
         </is>
       </c>
       <c r="L16" s="18">
-        <f>L151</f>
+        <f>L152</f>
         <v/>
       </c>
       <c r="M16" s="20" t="n"/>
       <c r="N16" s="5">
-        <f>N151</f>
+        <f>N152</f>
         <v/>
       </c>
       <c r="O16" s="3" t="inlineStr">
@@ -2090,7 +2090,7 @@
         </is>
       </c>
       <c r="L17" s="18">
-        <f>L161</f>
+        <f>L162</f>
         <v/>
       </c>
       <c r="M17" s="20" t="n"/>
@@ -2565,7 +2565,7 @@
         </is>
       </c>
       <c r="L46" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
@@ -2574,66 +2574,65 @@
       </c>
       <c r="O46" s="3" t="inlineStr">
         <is>
-          <t>Diâmetro do furo do aparelho (chumbador).</t>
+          <t>Diâmetro de cada furo do aparelho (chumbador).</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="K47" s="1" t="inlineStr">
         <is>
+          <t>n,furos</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="O47" s="3" t="inlineStr">
+        <is>
+          <t>Furos em cada aparelho (cada viga). Total = 2 aparelhos × n,furos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="K48" s="1" t="inlineStr">
+        <is>
           <t>σ,lim</t>
         </is>
       </c>
-      <c r="L47" s="4" t="n">
+      <c r="L48" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="M47" s="2" t="inlineStr">
+      <c r="M48" s="2" t="inlineStr">
         <is>
           <t>MPa</t>
         </is>
       </c>
-      <c r="O47" s="3" t="inlineStr">
+      <c r="O48" s="3" t="inlineStr">
         <is>
           <t>Tensão limite no aparelho de apoio (dado do fabricante).</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="K48" s="12" t="inlineStr">
+    <row r="49">
+      <c r="K49" s="12" t="inlineStr">
         <is>
           <t>1.6 Cargas</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="K49" s="1" t="inlineStr">
-        <is>
-          <t>Nk</t>
-        </is>
-      </c>
-      <c r="L49" s="9">
-        <f>2903.585/1.4</f>
-        <v/>
-      </c>
-      <c r="M49" s="2" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-      <c r="O49" s="3" t="inlineStr">
-        <is>
-          <t>Força normal característica transmitida pela viga.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="K50" s="1" t="inlineStr">
         <is>
-          <t>Nd</t>
-        </is>
-      </c>
-      <c r="L50" s="6">
-        <f>L49*L22</f>
+          <t>Nk</t>
+        </is>
+      </c>
+      <c r="L50" s="9">
+        <f>2903.585/1.4</f>
         <v/>
       </c>
       <c r="M50" s="2" t="inlineStr">
@@ -2643,41 +2642,40 @@
       </c>
       <c r="O50" s="3" t="inlineStr">
         <is>
-          <t>Força normal de cálculo.</t>
+          <t>Força normal característica transmitida pela viga.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="K51" s="1" t="inlineStr">
         <is>
-          <t>H?</t>
-        </is>
-      </c>
-      <c r="L51" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
+          <t>Nd</t>
+        </is>
+      </c>
+      <c r="L51" s="6">
+        <f>L50*L22</f>
+        <v/>
       </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>kN</t>
         </is>
       </c>
       <c r="O51" s="3" t="inlineStr">
         <is>
-          <t>Considerar força horizontal da viga? (Sim/Não)</t>
+          <t>Força normal de cálculo.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="K52" s="1" t="inlineStr">
         <is>
-          <t>Apoio</t>
+          <t>H?</t>
         </is>
       </c>
       <c r="L52" s="4" t="inlineStr">
         <is>
-          <t>Elastômero</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr">
@@ -2687,19 +2685,20 @@
       </c>
       <c r="O52" s="3" t="inlineStr">
         <is>
-          <t>Tipo de apoio: define μ pela tabela abaixo.</t>
+          <t>Considerar força horizontal da viga? (Sim/Não)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="K53" s="1" t="inlineStr">
         <is>
-          <t>μ</t>
-        </is>
-      </c>
-      <c r="L53" s="22">
-        <f>IFERROR(INDEX($L$57:$L$62,MATCH(L52,$O$57:$O$62,0)),0)</f>
-        <v/>
+          <t>Apoio</t>
+        </is>
+      </c>
+      <c r="L53" s="4" t="inlineStr">
+        <is>
+          <t>Elastômero</t>
+        </is>
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
@@ -2708,39 +2707,39 @@
       </c>
       <c r="O53" s="3" t="inlineStr">
         <is>
-          <t>Coeficiente de atrito do tipo de apoio (tabela abaixo).</t>
+          <t>Tipo de apoio: define μ pela tabela abaixo.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="K54" s="1" t="inlineStr">
         <is>
-          <t>Hk</t>
-        </is>
-      </c>
-      <c r="L54" s="6">
-        <f>IF(L51="Sim",L53*L49,0)</f>
+          <t>μ</t>
+        </is>
+      </c>
+      <c r="L54" s="22">
+        <f>IFERROR(INDEX($L$58:$L$63,MATCH(L53,$O$58:$O$63,0)),0)</f>
         <v/>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>kN</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O54" s="3" t="inlineStr">
         <is>
-          <t>Força horizontal característica (μ·Nk).</t>
+          <t>Coeficiente de atrito do tipo de apoio (tabela abaixo).</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="K55" s="1" t="inlineStr">
         <is>
-          <t>Hd</t>
+          <t>Hk</t>
         </is>
       </c>
       <c r="L55" s="6">
-        <f>L54*L22</f>
+        <f>IF(L52="Sim",L54*L50,0)</f>
         <v/>
       </c>
       <c r="M55" s="2" t="inlineStr">
@@ -2750,46 +2749,52 @@
       </c>
       <c r="O55" s="3" t="inlineStr">
         <is>
-          <t>Força horizontal de cálculo.</t>
+          <t>Força horizontal característica (μ·Nk).</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="K56" s="1" t="inlineStr">
         <is>
+          <t>Hd</t>
+        </is>
+      </c>
+      <c r="L56" s="6">
+        <f>L55*L22</f>
+        <v/>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>kN</t>
+        </is>
+      </c>
+      <c r="O56" s="3" t="inlineStr">
+        <is>
+          <t>Força horizontal de cálculo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="K57" s="1" t="inlineStr">
+        <is>
           <t>Tabela μ</t>
         </is>
       </c>
-      <c r="L56" s="17" t="inlineStr">
+      <c r="L57" s="17" t="inlineStr">
         <is>
           <t>μ</t>
         </is>
       </c>
-      <c r="M56" s="17" t="n"/>
-      <c r="O56" s="12" t="inlineStr">
+      <c r="M57" s="17" t="n"/>
+      <c r="O57" s="12" t="inlineStr">
         <is>
           <t>Tipo de apoio (escolha em "Apoio")</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="L57" s="9" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="M57" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O57" s="3" t="inlineStr">
-        <is>
-          <t>Juntas a seco</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="L58" s="9" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
@@ -2798,13 +2803,13 @@
       </c>
       <c r="O58" s="3" t="inlineStr">
         <is>
-          <t>Argamassa</t>
+          <t>Juntas a seco</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="L59" s="9" t="n">
-        <v>0.16</v>
+        <v>0.5</v>
       </c>
       <c r="M59" s="2" t="inlineStr">
         <is>
@@ -2813,13 +2818,13 @@
       </c>
       <c r="O59" s="3" t="inlineStr">
         <is>
-          <t>Elastômero</t>
+          <t>Argamassa</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="L60" s="9" t="n">
-        <v>0.08</v>
+        <v>0.16</v>
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
@@ -2828,13 +2833,13 @@
       </c>
       <c r="O60" s="3" t="inlineStr">
         <is>
-          <t>Politetrafluoretileno</t>
+          <t>Elastômero</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="L61" s="9" t="n">
-        <v>0.25</v>
+        <v>0.08</v>
       </c>
       <c r="M61" s="2" t="inlineStr">
         <is>
@@ -2843,91 +2848,84 @@
       </c>
       <c r="O61" s="3" t="inlineStr">
         <is>
-          <t>Chapas metálicas não soldadas</t>
+          <t>Politetrafluoretileno</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="L62" s="9" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O62" s="3" t="inlineStr">
+        <is>
+          <t>Chapas metálicas não soldadas</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="L63" s="9" t="n">
         <v>0.4</v>
       </c>
-      <c r="M62" s="2" t="inlineStr">
+      <c r="M63" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O62" s="3" t="inlineStr">
+      <c r="O63" s="3" t="inlineStr">
         <is>
           <t>Concreto x chapa metálica</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="K63" s="12" t="inlineStr">
+    <row r="64" s="15">
+      <c r="K64" s="12" t="inlineStr">
         <is>
           <t>1.7 Modelo de cálculo – bloco parcialmente carregado × consolo</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="78" customHeight="1" s="15">
-      <c r="K64" s="14" t="inlineStr">
+    <row r="65" ht="78" customHeight="1" s="15">
+      <c r="K65" s="14" t="inlineStr">
         <is>
           <t>BLOCO: o aparelho fica todo sobre o pilar (x,ap ≤ 0). A carga desce e se ESPALHA para a seção do pilar → compressão sob o apoio + fendilhamento (item 2), tirante do topo pela referência (item 3). As mísulas não recebem carga.   CONSOLO: parte do aparelho fica fora da face do pilar (x,ap &gt; 0). Essa parte está pendurada na mísula e só chega ao pilar por biela + tirante (NBR 9062, item 4) – vale mesmo para consolo muito curto (a/d ≤ 0,5). Na direção h a carga CONVERGE para o pilar (não espalha), então ali não existe bloco: tirante e costura são do consolo; o fendilhamento de bloco só é verificado na direção b (b0 → b).</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="K65" s="1" t="inlineStr">
-        <is>
-          <t>x,ap</t>
-        </is>
-      </c>
-      <c r="L65" s="23">
-        <f>L37/2-L32/2-L42</f>
-        <v/>
-      </c>
-      <c r="M65" s="2" t="inlineStr">
-        <is>
-          <t>cm</t>
-        </is>
-      </c>
-      <c r="O65" s="3" t="inlineStr">
-        <is>
-          <t>a,cab/2 − h,pil/2 − F,ap: quanto a borda externa do aparelho passa da face do pilar. ≤ 0 → todo sobre o pilar.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="K66" s="1" t="inlineStr">
         <is>
-          <t>Indicado</t>
-        </is>
-      </c>
-      <c r="L66" s="18">
-        <f>IF(L65&lt;=0,"Bloco","Consolo")</f>
+          <t>x,ap</t>
+        </is>
+      </c>
+      <c r="L66" s="23">
+        <f>L37/2-L32/2-L42</f>
         <v/>
       </c>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>cm</t>
         </is>
       </c>
       <c r="O66" s="3" t="inlineStr">
         <is>
-          <t>Modelo indicado pela geometria: x,ap ≤ 0 → Bloco; x,ap &gt; 0 → Consolo.</t>
+          <t>a,cab/2 − h,pil/2 − F,ap: quanto a borda externa do aparelho passa da face do pilar. ≤ 0 → todo sobre o pilar.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="K67" s="1" t="inlineStr">
         <is>
-          <t>Escolha</t>
-        </is>
-      </c>
-      <c r="L67" s="4" t="inlineStr">
-        <is>
-          <t>Automático</t>
-        </is>
+          <t>Indicado</t>
+        </is>
+      </c>
+      <c r="L67" s="18">
+        <f>IF(L66&lt;=0,"Bloco","Consolo")</f>
+        <v/>
       </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
@@ -2936,198 +2934,199 @@
       </c>
       <c r="O67" s="3" t="inlineStr">
         <is>
-          <t>Automático (recomendado) ou forçar "Bloco" / "Consolo".</t>
+          <t>Modelo indicado pela geometria: x,ap ≤ 0 → Bloco; x,ap &gt; 0 → Consolo.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="K68" s="1" t="inlineStr">
         <is>
+          <t>Escolha</t>
+        </is>
+      </c>
+      <c r="L68" s="4" t="inlineStr">
+        <is>
+          <t>Automático</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O68" s="3" t="inlineStr">
+        <is>
+          <t>Automático (recomendado) ou forçar "Bloco" / "Consolo".</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="K69" s="1" t="inlineStr">
+        <is>
           <t>Modelo</t>
         </is>
       </c>
-      <c r="L68" s="18">
-        <f>IF(L67="Automático",L66,L67)</f>
-        <v/>
-      </c>
-      <c r="M68" s="2" t="inlineStr">
+      <c r="L69" s="18">
+        <f>IF(L68="Automático",L67,L68)</f>
+        <v/>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N68" s="5">
-        <f>IF(L68=L66,"Ok",IF(L68="Bloco","Inseguro: carga fora do pilar – usar Consolo","Mísula sem carga – usar Bloco"))</f>
-        <v/>
-      </c>
-      <c r="O68" s="3" t="inlineStr">
+      <c r="N69" s="5">
+        <f>IF(L69=L67,"Ok",IF(L69="Bloco","Inseguro: carga fora do pilar – usar Consolo","Mísula sem carga – usar Bloco"))</f>
+        <v/>
+      </c>
+      <c r="O69" s="3" t="inlineStr">
         <is>
           <t>Modelo adotado: define as armaduras calculadas e o desenho.</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="48" customHeight="1" s="15">
-      <c r="K69" s="21">
-        <f>IF(L68="Bloco","⚠ BLOCO PARCIALMENTE CARREGADO – aparelho todo sobre o pilar. Armaduras: cintas de fendilhamento (item 2: direções h e b + regra 0,25·Nd da referência), tirante do topo pela referência (item 3.1) e parede oposta (3.2). O consolo (item 4) não se aplica: sem costura.",IF(L65&lt;=0,"⚠ CONSOLO forçado, mas o aparelho não passa da face do pilar: a mísula não recebe carga – use o modelo Bloco.","⚠ CONSOLO – o aparelho passa "&amp;ROUND(L65,1)&amp;" cm da face do pilar de cada lado: a mísula é um consolo "&amp;LOWER(L129)&amp;" (a/d = "&amp;ROUND(L128,2)&amp;"). Armaduras: tirante do topo e costura pelo consolo (item 4, NBR 9062); cintas de fendilhamento só na direção b (b0 → b), pois na direção h a carga converge para o pilar e não espalha (item 2). Parede oposta (3.2) mantida."))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70"/>
+    <row r="70" ht="48" customHeight="1" s="15">
+      <c r="K70" s="21">
+        <f>IF(L69="Bloco","⚠ BLOCO PARCIALMENTE CARREGADO – aparelho todo sobre o pilar. Armaduras: cintas de fendilhamento (item 2: direções h e b + regra 0,25·Nd da referência), tirante do topo pela referência (item 3.1) e parede oposta (3.2). O consolo (item 4) não se aplica: sem costura.",IF(L66&lt;=0,"⚠ CONSOLO forçado, mas o aparelho não passa da face do pilar: a mísula não recebe carga – use o modelo Bloco.","⚠ CONSOLO – o aparelho passa "&amp;ROUND(L66,1)&amp;" cm da face do pilar de cada lado: a mísula é um consolo "&amp;LOWER(L130)&amp;" (a/d = "&amp;ROUND(L129,2)&amp;"). Armaduras: tirante do topo e costura pelo consolo (item 4, NBR 9062); cintas de fendilhamento só na direção b (b0 → b), pois na direção h a carga converge para o pilar e não espalha (item 2). Parede oposta (3.2) mantida."))</f>
+        <v/>
+      </c>
+    </row>
     <row r="71"/>
-    <row r="72">
-      <c r="K72" s="16" t="inlineStr">
+    <row r="72"/>
+    <row r="73">
+      <c r="K73" s="16" t="inlineStr">
         <is>
           <t>2 . BLOCO PARCIALMENTE CARREGADO (região logo abaixo do aparelho)</t>
         </is>
       </c>
-      <c r="L72" s="19" t="n"/>
-      <c r="M72" s="19" t="n"/>
-      <c r="N72" s="19" t="n"/>
-      <c r="O72" s="19" t="n"/>
-      <c r="P72" s="19" t="n"/>
-      <c r="Q72" s="19" t="n"/>
-      <c r="R72" s="19" t="n"/>
-      <c r="S72" s="19" t="n"/>
-      <c r="T72" s="20" t="n"/>
-    </row>
-    <row r="73"/>
-    <row r="74" ht="48" customHeight="1" s="15">
-      <c r="K74" s="14" t="inlineStr">
+      <c r="L73" s="19" t="n"/>
+      <c r="M73" s="19" t="n"/>
+      <c r="N73" s="19" t="n"/>
+      <c r="O73" s="19" t="n"/>
+      <c r="P73" s="19" t="n"/>
+      <c r="Q73" s="19" t="n"/>
+      <c r="R73" s="19" t="n"/>
+      <c r="S73" s="19" t="n"/>
+      <c r="T73" s="20" t="n"/>
+    </row>
+    <row r="74"/>
+    <row r="75" ht="48" customHeight="1" s="15">
+      <c r="K75" s="14" t="inlineStr">
         <is>
           <t>A carga entra por uma área pequena (a0 × b0). Onde ela ESPALHA para uma seção maior surgem compressão sob o apoio (2.1) e tração transversal – fendilhamento (2.2 e 2.3), resistida por cintas a partir do topo. Cada direção é verificada: h (a0 → h,pil) e b (b0 → b). Se a0 ≥ h,pil a carga converge na direção h e ali não há fendilhamento (é o consolo do item 4). A regra 0,25·Nd da referência só entra no modelo Bloco.</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="K75" s="12" t="inlineStr">
+    <row r="76">
+      <c r="K76" s="12" t="inlineStr">
         <is>
           <t>2.1 Compressão sob o apoio (NBR 6118, 21.2.1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="K76" s="1" t="inlineStr">
-        <is>
-          <t>A0</t>
-        </is>
-      </c>
-      <c r="L76" s="6">
-        <f>L43*L44</f>
-        <v/>
-      </c>
-      <c r="M76" s="2" t="inlineStr">
-        <is>
-          <t>cm²</t>
-        </is>
-      </c>
-      <c r="O76" s="3" t="inlineStr">
-        <is>
-          <t>Área carregada (a0 × b0).</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="K77" s="1" t="inlineStr">
         <is>
-          <t>β</t>
-        </is>
-      </c>
-      <c r="L77" s="22">
-        <f>MIN(L37/L43,L33/L44,3.3)</f>
+          <t>A0</t>
+        </is>
+      </c>
+      <c r="L77" s="6">
+        <f>L43*L44</f>
         <v/>
       </c>
       <c r="M77" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>cm²</t>
         </is>
       </c>
       <c r="O77" s="3" t="inlineStr">
         <is>
-          <t>β = √(Ac1/Ac0), Ac1 homotética a A0 na cabeça (≤ 3,3).</t>
+          <t>Área carregada (a0 × b0).</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="K78" s="1" t="inlineStr">
         <is>
-          <t>β·fcd</t>
-        </is>
-      </c>
-      <c r="L78" s="6">
-        <f>L77*L27</f>
+          <t>β</t>
+        </is>
+      </c>
+      <c r="L78" s="22">
+        <f>MIN(L37/L43,L33/L44,3.3)</f>
         <v/>
       </c>
       <c r="M78" s="2" t="inlineStr">
         <is>
-          <t>MPa</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O78" s="3" t="inlineStr">
         <is>
-          <t>Tensão resistente sob o apoio.</t>
+          <t>β = √(Ac1/Ac0), Ac1 homotética a A0 na cabeça (≤ 3,3).</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="K79" s="1" t="inlineStr">
         <is>
+          <t>β·fcd</t>
+        </is>
+      </c>
+      <c r="L79" s="6">
+        <f>L78*L27</f>
+        <v/>
+      </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="O79" s="3" t="inlineStr">
+        <is>
+          <t>Tensão resistente sob o apoio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="K80" s="1" t="inlineStr">
+        <is>
           <t>σc</t>
         </is>
       </c>
-      <c r="L79" s="6">
-        <f>L50/L76*10</f>
-        <v/>
-      </c>
-      <c r="M79" s="2" t="inlineStr">
+      <c r="L80" s="6">
+        <f>L51/L77*10</f>
+        <v/>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
         <is>
           <t>MPa</t>
         </is>
       </c>
-      <c r="N79" s="5">
-        <f>IF(L79&lt;=L78,"Ok","Aumentar apoio ou fck")</f>
-        <v/>
-      </c>
-      <c r="O79" s="3" t="inlineStr">
+      <c r="N80" s="5">
+        <f>IF(L80&lt;=L79,"Ok","Aumentar apoio ou fck")</f>
+        <v/>
+      </c>
+      <c r="O80" s="3" t="inlineStr">
         <is>
           <t>Tensão atuante sob o apoio (Nd/A0).</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="K80" s="12" t="inlineStr">
+    <row r="81">
+      <c r="K81" s="12" t="inlineStr">
         <is>
           <t>2.2 Tensão de tração transversal (necessidade de cintamento)</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="K81" s="1" t="inlineStr">
-        <is>
-          <t>σt,h</t>
-        </is>
-      </c>
-      <c r="L81" s="6">
-        <f>2.1*L49/(L32*L33)*MAX(0,1-L43/L32)*10</f>
-        <v/>
-      </c>
-      <c r="M81" s="2" t="inlineStr">
-        <is>
-          <t>MPa</t>
-        </is>
-      </c>
-      <c r="O81" s="3" t="inlineStr">
-        <is>
-          <t>Direção h: σt = 2,1·Nk/(h,pil·b)·(1−a0/h,pil). Zero se a0 ≥ h,pil (carga converge).</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="K82" s="1" t="inlineStr">
         <is>
-          <t>σt,b</t>
+          <t>σt,h</t>
         </is>
       </c>
       <c r="L82" s="6">
-        <f>2.1*L49/(L32*L33)*MAX(0,1-L44/L33)*10</f>
+        <f>2.1*L50/(L32*L33)*MAX(0,1-L43/L32)*10</f>
         <v/>
       </c>
       <c r="M82" s="2" t="inlineStr">
@@ -3137,18 +3136,18 @@
       </c>
       <c r="O82" s="3" t="inlineStr">
         <is>
-          <t>Direção b: σt = 2,1·Nk/(h,pil·b)·(1−b0/b).</t>
+          <t>Direção h: σt = 2,1·Nk/(h,pil·b)·(1−a0/h,pil). Zero se a0 ≥ h,pil (carga converge).</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="K83" s="1" t="inlineStr">
         <is>
-          <t>σt</t>
+          <t>σt,b</t>
         </is>
       </c>
       <c r="L83" s="6">
-        <f>MAX(L81,L82)</f>
+        <f>2.1*L50/(L32*L33)*MAX(0,1-L44/L33)*10</f>
         <v/>
       </c>
       <c r="M83" s="2" t="inlineStr">
@@ -3158,71 +3157,71 @@
       </c>
       <c r="O83" s="3" t="inlineStr">
         <is>
-          <t>Maior das duas direções (compara com fctk/2).</t>
+          <t>Direção b: σt = 2,1·Nk/(h,pil·b)·(1−b0/b).</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="K84" s="1" t="inlineStr">
         <is>
+          <t>σt</t>
+        </is>
+      </c>
+      <c r="L84" s="6">
+        <f>MAX(L82,L83)</f>
+        <v/>
+      </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="O84" s="3" t="inlineStr">
+        <is>
+          <t>Maior das duas direções (compara com fctk/2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="K85" s="1" t="inlineStr">
+        <is>
           <t>fctk/2</t>
         </is>
       </c>
-      <c r="L84" s="6">
+      <c r="L85" s="6">
         <f>0.7*0.3*L26^(2/3)/2</f>
         <v/>
       </c>
-      <c r="M84" s="2" t="inlineStr">
+      <c r="M85" s="2" t="inlineStr">
         <is>
           <t>MPa</t>
         </is>
       </c>
-      <c r="N84" s="5">
-        <f>IF(L83&lt;=L84,"Ok – cintas dispensáveis","Calcular cintamento")</f>
-        <v/>
-      </c>
-      <c r="O84" s="3" t="inlineStr">
+      <c r="N85" s="5">
+        <f>IF(L84&lt;=L85,"Ok – cintas dispensáveis","Calcular cintamento")</f>
+        <v/>
+      </c>
+      <c r="O85" s="3" t="inlineStr">
         <is>
           <t>Limite para dispensar cintas: fctk,inf/2.</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="K85" s="12" t="inlineStr">
+    <row r="86">
+      <c r="K86" s="12" t="inlineStr">
         <is>
           <t>2.3 Armadura de fendilhamento (cintamento)</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="K86" s="1" t="inlineStr">
-        <is>
-          <t>Fad,h</t>
-        </is>
-      </c>
-      <c r="L86" s="6">
-        <f>0.3*L50*MAX(0,1-L43/L32)</f>
-        <v/>
-      </c>
-      <c r="M86" s="2" t="inlineStr">
-        <is>
-          <t>kN</t>
-        </is>
-      </c>
-      <c r="O86" s="3" t="inlineStr">
-        <is>
-          <t>Direção h (NBR 6118): 0,3·Nd·(1−a0/h,pil). Zero se a0 ≥ h,pil.</t>
         </is>
       </c>
     </row>
     <row r="87" s="15">
       <c r="K87" s="1" t="inlineStr">
         <is>
-          <t>Fad,b</t>
+          <t>Fad,h</t>
         </is>
       </c>
       <c r="L87" s="6">
-        <f>0.3*L50*MAX(0,1-L44/L33)</f>
+        <f>0.3*L51*MAX(0,1-L43/L32)</f>
         <v/>
       </c>
       <c r="M87" s="2" t="inlineStr">
@@ -3232,18 +3231,18 @@
       </c>
       <c r="O87" s="3" t="inlineStr">
         <is>
-          <t>Direção b (NBR 6118): 0,3·Nd·(1−b0/b).</t>
+          <t>Direção h (NBR 6118): 0,3·Nd·(1−a0/h,pil). Zero se a0 ≥ h,pil.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="K88" s="1" t="inlineStr">
         <is>
-          <t>Fad,NBR</t>
+          <t>Fad,b</t>
         </is>
       </c>
       <c r="L88" s="6">
-        <f>MAX(L86,L87)</f>
+        <f>0.3*L51*MAX(0,1-L44/L33)</f>
         <v/>
       </c>
       <c r="M88" s="2" t="inlineStr">
@@ -3253,18 +3252,18 @@
       </c>
       <c r="O88" s="3" t="inlineStr">
         <is>
-          <t>Força de fendilhamento pela NBR 6118 (maior direção).</t>
+          <t>Direção b (NBR 6118): 0,3·Nd·(1−b0/b).</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="K89" s="1" t="inlineStr">
         <is>
-          <t>Fad,ref</t>
+          <t>Fad,NBR</t>
         </is>
       </c>
       <c r="L89" s="6">
-        <f>0.25*L50+0.25*L55</f>
+        <f>MAX(L87,L88)</f>
         <v/>
       </c>
       <c r="M89" s="2" t="inlineStr">
@@ -3274,18 +3273,18 @@
       </c>
       <c r="O89" s="3" t="inlineStr">
         <is>
-          <t>Planilha de referência: 0,25·Nd + 0,25·Hd (só no modelo Bloco).</t>
+          <t>Força de fendilhamento pela NBR 6118 (maior direção).</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="K90" s="1" t="inlineStr">
         <is>
-          <t>Fad</t>
+          <t>Fad,ref</t>
         </is>
       </c>
       <c r="L90" s="6">
-        <f>IF(L68="Bloco",MAX(L88,L89),L88)</f>
+        <f>0.25*L51+0.25*L56</f>
         <v/>
       </c>
       <c r="M90" s="2" t="inlineStr">
@@ -3295,219 +3294,219 @@
       </c>
       <c r="O90" s="3" t="inlineStr">
         <is>
-          <t>Força adotada: Bloco = maior das duas; Consolo = só a NBR.</t>
+          <t>Planilha de referência: 0,25·Nd + 0,25·Hd (só no modelo Bloco).</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="K91" s="1" t="inlineStr">
         <is>
-          <t>As,fend</t>
+          <t>Fad</t>
         </is>
       </c>
       <c r="L91" s="6">
-        <f>L90/L29</f>
+        <f>IF(L69="Bloco",MAX(L89,L90),L89)</f>
         <v/>
       </c>
       <c r="M91" s="2" t="inlineStr">
         <is>
-          <t>cm²</t>
+          <t>kN</t>
         </is>
       </c>
       <c r="O91" s="3" t="inlineStr">
         <is>
-          <t>Área de aço necessária para o fendilhamento.</t>
+          <t>Força adotada: Bloco = maior das duas; Consolo = só a NBR.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="K92" s="1" t="inlineStr">
         <is>
-          <t>k,dist</t>
-        </is>
-      </c>
-      <c r="L92" s="4" t="n">
-        <v>0.6</v>
+          <t>As,fend</t>
+        </is>
+      </c>
+      <c r="L92" s="6">
+        <f>L91/L29</f>
+        <v/>
       </c>
       <c r="M92" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>cm²</t>
         </is>
       </c>
       <c r="O92" s="3" t="inlineStr">
         <is>
-          <t>Fração do lado do pilar para distribuir as cintas (0,6·a).</t>
+          <t>Área de aço necessária para o fendilhamento.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="K93" s="1" t="inlineStr">
         <is>
-          <t>dist</t>
-        </is>
-      </c>
-      <c r="L93" s="6">
-        <f>L92*IF(L68="Bloco",MAX(L32,L33),L33)</f>
-        <v/>
+          <t>k,dist</t>
+        </is>
+      </c>
+      <c r="L93" s="4" t="n">
+        <v>0.6</v>
       </c>
       <c r="M93" s="2" t="inlineStr">
         <is>
-          <t>cm</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O93" s="3" t="inlineStr">
         <is>
-          <t>Altura das cintas a partir do topo: 0,6·maior lado do pilar (Bloco) ou 0,6·b (Consolo).</t>
+          <t>Fração do lado do pilar para distribuir as cintas (0,6·a).</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="K94" s="1" t="inlineStr">
         <is>
-          <t>Ø</t>
-        </is>
-      </c>
-      <c r="L94" s="4" t="n">
-        <v>12.5</v>
+          <t>dist</t>
+        </is>
+      </c>
+      <c r="L94" s="6">
+        <f>L93*IF(L69="Bloco",MAX(L32,L33),L33)</f>
+        <v/>
       </c>
       <c r="M94" s="2" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>cm</t>
         </is>
       </c>
       <c r="O94" s="3" t="inlineStr">
         <is>
-          <t>Bitola escolhida para as cintas.</t>
+          <t>Altura das cintas a partir do topo: 0,6·maior lado do pilar (Bloco) ou 0,6·b (Consolo).</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="K95" s="1" t="inlineStr">
         <is>
-          <t>ramos</t>
+          <t>Ø</t>
         </is>
       </c>
       <c r="L95" s="4" t="n">
-        <v>2</v>
+        <v>12.5</v>
       </c>
       <c r="M95" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="O95" s="3" t="inlineStr">
         <is>
-          <t>Ramos de cada cinta (estribo fechado = 2).</t>
+          <t>Bitola escolhida para as cintas.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="K96" s="1" t="inlineStr">
         <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="L96" s="7">
-        <f>MAX(2,ROUNDUP(L91/(L95*PI()*(L94/10)^2/4),0))</f>
-        <v/>
+          <t>ramos</t>
+        </is>
+      </c>
+      <c r="L96" s="4" t="n">
+        <v>2</v>
       </c>
       <c r="M96" s="2" t="inlineStr">
         <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="N96" s="5">
-        <f>IF(L96*L95*PI()*(L94/10)^2/4&lt;L91,"Rever",IF(L97&lt;5,"s &lt; 5 cm – aumentar Ø ou ramos","Ok"))</f>
-        <v/>
+          <t>-</t>
+        </is>
       </c>
       <c r="O96" s="3" t="inlineStr">
         <is>
-          <t>Quantidade de cintas necessárias (mínimo 2).</t>
+          <t>Ramos de cada cinta (estribo fechado = 2).</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="K97" s="1" t="inlineStr">
         <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="L97" s="7">
+        <f>MAX(2,ROUNDUP(L92/(L96*PI()*(L95/10)^2/4),0))</f>
+        <v/>
+      </c>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="N97" s="5">
+        <f>IF(L97*L96*PI()*(L95/10)^2/4&lt;L92,"Rever",IF(L98&lt;5,"s &lt; 5 cm – aumentar Ø ou ramos","Ok"))</f>
+        <v/>
+      </c>
+      <c r="O97" s="3" t="inlineStr">
+        <is>
+          <t>Quantidade de cintas necessárias (mínimo 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="K98" s="1" t="inlineStr">
+        <is>
           <t>s</t>
         </is>
       </c>
-      <c r="L97" s="7">
-        <f>ROUNDDOWN(L93/L96,0)</f>
-        <v/>
-      </c>
-      <c r="M97" s="2" t="inlineStr">
+      <c r="L98" s="7">
+        <f>ROUNDDOWN(L94/L97,0)</f>
+        <v/>
+      </c>
+      <c r="M98" s="2" t="inlineStr">
         <is>
           <t>cm</t>
         </is>
       </c>
-      <c r="O97" s="3" t="inlineStr">
+      <c r="O98" s="3" t="inlineStr">
         <is>
           <t>Espaçamento das cintas dentro de dist.</t>
         </is>
       </c>
     </row>
-    <row r="98"/>
-    <row r="99">
-      <c r="K99" s="16" t="inlineStr">
+    <row r="99"/>
+    <row r="100">
+      <c r="K100" s="16" t="inlineStr">
         <is>
           <t>3 . TIRANTES NO TOPO DA CABEÇA (planilha de referência)</t>
         </is>
       </c>
-      <c r="L99" s="19" t="n"/>
-      <c r="M99" s="19" t="n"/>
-      <c r="N99" s="19" t="n"/>
-      <c r="O99" s="19" t="n"/>
-      <c r="P99" s="19" t="n"/>
-      <c r="Q99" s="19" t="n"/>
-      <c r="R99" s="19" t="n"/>
-      <c r="S99" s="19" t="n"/>
-      <c r="T99" s="20" t="n"/>
-    </row>
-    <row r="100"/>
-    <row r="101" ht="32.1" customHeight="1" s="15">
-      <c r="K101" s="14" t="inlineStr">
+      <c r="L100" s="19" t="n"/>
+      <c r="M100" s="19" t="n"/>
+      <c r="N100" s="19" t="n"/>
+      <c r="O100" s="19" t="n"/>
+      <c r="P100" s="19" t="n"/>
+      <c r="Q100" s="19" t="n"/>
+      <c r="R100" s="19" t="n"/>
+      <c r="S100" s="19" t="n"/>
+      <c r="T100" s="20" t="n"/>
+    </row>
+    <row r="101"/>
+    <row r="102" ht="32.1" customHeight="1" s="15">
+      <c r="K102" s="14" t="inlineStr">
         <is>
           <t>Barras horizontais logo abaixo do topo. Modelo BLOCO: tirante pela regra da referência (0,25·Nd + 1,8·Hd). Modelo CONSOLO: o tirante da face carregada é o tirante do consolo (item 4) – usa-se o maior entre o consolo e a armadura mínima.</t>
         </is>
       </c>
     </row>
-    <row r="102" s="15">
-      <c r="K102" s="12" t="inlineStr">
+    <row r="103">
+      <c r="K103" s="12" t="inlineStr">
         <is>
           <t>3.1 Tirante da face carregada</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="K103" s="1" t="inlineStr">
-        <is>
-          <t>As,ref</t>
-        </is>
-      </c>
-      <c r="L103" s="6">
-        <f>(0.25*L50+1.8*L55)/L29</f>
-        <v/>
-      </c>
-      <c r="M103" s="2" t="inlineStr">
-        <is>
-          <t>cm²</t>
-        </is>
-      </c>
-      <c r="O103" s="3" t="inlineStr">
-        <is>
-          <t>Referência: (0,25·Nd + 1,8·Hd)/fyd – modelo Bloco.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="K104" s="1" t="inlineStr">
         <is>
-          <t>As,cons</t>
+          <t>As,ref</t>
         </is>
       </c>
       <c r="L104" s="6">
-        <f>L135</f>
+        <f>(0.25*L51+1.8*L56)/L29</f>
         <v/>
       </c>
       <c r="M104" s="2" t="inlineStr">
@@ -3517,14 +3516,14 @@
       </c>
       <c r="O104" s="3" t="inlineStr">
         <is>
-          <t>Tirante exigido pelo consolo (item 4.3) – modelo Consolo.</t>
+          <t>Referência: (0,25·Nd + 1,8·Hd)/fyd – modelo Bloco.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="K105" s="1" t="inlineStr">
         <is>
-          <t>As,mín</t>
+          <t>As,cons</t>
         </is>
       </c>
       <c r="L105" s="6">
@@ -3538,18 +3537,18 @@
       </c>
       <c r="O105" s="3" t="inlineStr">
         <is>
-          <t>Armadura mínima do tirante do consolo – modelo Consolo.</t>
+          <t>Tirante exigido pelo consolo (item 4.3) – modelo Consolo.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="K106" s="1" t="inlineStr">
         <is>
-          <t>As,tir</t>
+          <t>As,mín</t>
         </is>
       </c>
       <c r="L106" s="6">
-        <f>IF(L68="Bloco",L103,MAX(L104,L105))</f>
+        <f>L137</f>
         <v/>
       </c>
       <c r="M106" s="2" t="inlineStr">
@@ -3559,189 +3558,189 @@
       </c>
       <c r="O106" s="3" t="inlineStr">
         <is>
-          <t>Área do tirante: Bloco = As,ref; Consolo = maior entre As,cons e As,mín.</t>
+          <t>Armadura mínima do tirante do consolo – modelo Consolo.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="K107" s="1" t="inlineStr">
         <is>
-          <t>Ø</t>
-        </is>
-      </c>
-      <c r="L107" s="4" t="n">
-        <v>25</v>
+          <t>As,tir</t>
+        </is>
+      </c>
+      <c r="L107" s="6">
+        <f>IF(L69="Bloco",L104,MAX(L105,L106))</f>
+        <v/>
       </c>
       <c r="M107" s="2" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>cm²</t>
         </is>
       </c>
       <c r="O107" s="3" t="inlineStr">
         <is>
-          <t>Bitola escolhida para o tirante.</t>
+          <t>Área do tirante: Bloco = As,ref; Consolo = maior entre As,cons e As,mín.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="K108" s="1" t="inlineStr">
         <is>
+          <t>Ø</t>
+        </is>
+      </c>
+      <c r="L108" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="O108" s="3" t="inlineStr">
+        <is>
+          <t>Bitola escolhida para o tirante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="K109" s="1" t="inlineStr">
+        <is>
           <t>n</t>
         </is>
       </c>
-      <c r="L108" s="7">
-        <f>MAX(2,ROUNDUP(L106/(PI()*(L107/10)^2/4),0))</f>
-        <v/>
-      </c>
-      <c r="M108" s="2" t="inlineStr">
+      <c r="L109" s="7">
+        <f>MAX(2,ROUNDUP(L107/(PI()*(L108/10)^2/4),0))</f>
+        <v/>
+      </c>
+      <c r="M109" s="2" t="inlineStr">
         <is>
           <t>un</t>
         </is>
       </c>
-      <c r="N108" s="5">
+      <c r="N109" s="5">
         <f>"Ok"</f>
         <v/>
       </c>
-      <c r="O108" s="3" t="inlineStr">
+      <c r="O109" s="3" t="inlineStr">
         <is>
           <t>Quantidade de barras do tirante (mínimo 2).</t>
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="K109" s="12" t="inlineStr">
+    <row r="110">
+      <c r="K110" s="12" t="inlineStr">
         <is>
           <t>3.2 Parede oposta</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="K110" s="1" t="inlineStr">
-        <is>
-          <t>As,par</t>
-        </is>
-      </c>
-      <c r="L110" s="6">
-        <f>(0.25*L50+2.5*L55)/L29</f>
-        <v/>
-      </c>
-      <c r="M110" s="2" t="inlineStr">
-        <is>
-          <t>cm²</t>
-        </is>
-      </c>
-      <c r="O110" s="3" t="inlineStr">
-        <is>
-          <t>Referência: (0,25·Nd + 2,5·Hd)/fyd.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="K111" s="1" t="inlineStr">
         <is>
-          <t>Ø</t>
-        </is>
-      </c>
-      <c r="L111" s="4" t="n">
-        <v>20</v>
+          <t>As,par</t>
+        </is>
+      </c>
+      <c r="L111" s="6">
+        <f>(0.25*L51+2.5*L56)/L29</f>
+        <v/>
       </c>
       <c r="M111" s="2" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>cm²</t>
         </is>
       </c>
       <c r="O111" s="3" t="inlineStr">
         <is>
-          <t>Bitola escolhida para a parede oposta.</t>
+          <t>Referência: (0,25·Nd + 2,5·Hd)/fyd.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="K112" s="1" t="inlineStr">
         <is>
+          <t>Ø</t>
+        </is>
+      </c>
+      <c r="L112" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="M112" s="2" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="O112" s="3" t="inlineStr">
+        <is>
+          <t>Bitola escolhida para a parede oposta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="K113" s="1" t="inlineStr">
+        <is>
           <t>n</t>
         </is>
       </c>
-      <c r="L112" s="7">
-        <f>MAX(2,ROUNDUP(L110/(PI()*(L111/10)^2/4),0))</f>
-        <v/>
-      </c>
-      <c r="M112" s="2" t="inlineStr">
+      <c r="L113" s="7">
+        <f>MAX(2,ROUNDUP(L111/(PI()*(L112/10)^2/4),0))</f>
+        <v/>
+      </c>
+      <c r="M113" s="2" t="inlineStr">
         <is>
           <t>un</t>
         </is>
       </c>
-      <c r="N112" s="5">
+      <c r="N113" s="5">
         <f>"Ok"</f>
         <v/>
       </c>
-      <c r="O112" s="3" t="inlineStr">
+      <c r="O113" s="3" t="inlineStr">
         <is>
           <t>Quantidade de barras da parede oposta (mínimo 2).</t>
         </is>
       </c>
     </row>
-    <row r="113"/>
-    <row r="114">
-      <c r="K114" s="16" t="inlineStr">
+    <row r="114"/>
+    <row r="115">
+      <c r="K115" s="16" t="inlineStr">
         <is>
           <t>4 . CABEÇA COM MÍSULA – CONSOLO (NBR 9062, consolos)</t>
         </is>
       </c>
-      <c r="L114" s="19" t="n"/>
-      <c r="M114" s="19" t="n"/>
-      <c r="N114" s="19" t="n"/>
-      <c r="O114" s="19" t="n"/>
-      <c r="P114" s="19" t="n"/>
-      <c r="Q114" s="19" t="n"/>
-      <c r="R114" s="19" t="n"/>
-      <c r="S114" s="19" t="n"/>
-      <c r="T114" s="20" t="n"/>
-    </row>
-    <row r="115"/>
-    <row r="116" ht="60" customHeight="1" s="15">
-      <c r="K116" s="14" t="inlineStr">
+      <c r="L115" s="19" t="n"/>
+      <c r="M115" s="19" t="n"/>
+      <c r="N115" s="19" t="n"/>
+      <c r="O115" s="19" t="n"/>
+      <c r="P115" s="19" t="n"/>
+      <c r="Q115" s="19" t="n"/>
+      <c r="R115" s="19" t="n"/>
+      <c r="S115" s="19" t="n"/>
+      <c r="T115" s="20" t="n"/>
+    </row>
+    <row r="116"/>
+    <row r="117" ht="60" customHeight="1" s="15">
+      <c r="K117" s="14" t="inlineStr">
         <is>
           <t>Aplica-se só no modelo CONSOLO (item 1.7). A cabeça é mais larga que o pilar: o trecho do aparelho que fica fora da face do pilar apoia-se num balanço (a mísula). Esse balanço trabalha como consolo – biela inclinada até o pilar e tirante no topo. O tipo depende de a/d: muito curto (a/d ≤ 0,5), curto (0,5 &lt; a/d ≤ 1) ou viga em balanço (a/d &gt; 1). Só UMA das três fórmulas é usada, conforme o tipo.</t>
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="K117" s="12" t="inlineStr">
+    <row r="118">
+      <c r="K118" s="12" t="inlineStr">
         <is>
           <t>4.1 Geometria da cabeça</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="K118" s="1" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="L118" s="6">
-        <f>MAX(0,(L37-L32)/2)</f>
-        <v/>
-      </c>
-      <c r="M118" s="2" t="inlineStr">
-        <is>
-          <t>cm</t>
-        </is>
-      </c>
-      <c r="O118" s="3" t="inlineStr">
-        <is>
-          <t>Projeção de cada mísula além da face do pilar.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="K119" s="1" t="inlineStr">
         <is>
-          <t>h,mís</t>
+          <t>p</t>
         </is>
       </c>
       <c r="L119" s="6">
-        <f>L118*TAN(RADIANS(L38))</f>
+        <f>MAX(0,(L37-L32)/2)</f>
         <v/>
       </c>
       <c r="M119" s="2" t="inlineStr">
@@ -3751,18 +3750,18 @@
       </c>
       <c r="O119" s="3" t="inlineStr">
         <is>
-          <t>Altura da parte inclinada (p·tgθ).</t>
+          <t>Projeção de cada mísula além da face do pilar.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="K120" s="1" t="inlineStr">
         <is>
-          <t>H,cab</t>
+          <t>h,mís</t>
         </is>
       </c>
       <c r="L120" s="6">
-        <f>L39+L119</f>
+        <f>L119*TAN(RADIANS(L38))</f>
         <v/>
       </c>
       <c r="M120" s="2" t="inlineStr">
@@ -3772,18 +3771,18 @@
       </c>
       <c r="O120" s="3" t="inlineStr">
         <is>
-          <t>Altura total da cabeça junto à face do pilar (h1 + h,mís).</t>
+          <t>Altura da parte inclinada (p·tgθ).</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="K121" s="1" t="inlineStr">
         <is>
-          <t>h1,mín</t>
+          <t>H,cab</t>
         </is>
       </c>
       <c r="L121" s="6">
-        <f>L120/2</f>
+        <f>L39+L120</f>
         <v/>
       </c>
       <c r="M121" s="2" t="inlineStr">
@@ -3791,115 +3790,115 @@
           <t>cm</t>
         </is>
       </c>
-      <c r="N121" s="5">
-        <f>IF(L68&lt;&gt;"Consolo","Não se aplica (bloco)",IF(L39&gt;=L121,"Ok","Aumentar h1 para "&amp;ROUNDUP(L119,0)&amp;" cm"))</f>
-        <v/>
-      </c>
       <c r="O121" s="3" t="inlineStr">
         <is>
-          <t>NBR 9062: h1 ≥ metade de H,cab.</t>
+          <t>Altura total da cabeça junto à face do pilar (h1 + h,mís).</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="K122" s="1" t="inlineStr">
         <is>
+          <t>h1,mín</t>
+        </is>
+      </c>
+      <c r="L122" s="6">
+        <f>L121/2</f>
+        <v/>
+      </c>
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t>cm</t>
+        </is>
+      </c>
+      <c r="N122" s="5">
+        <f>IF(L69&lt;&gt;"Consolo","Não se aplica (bloco)",IF(L39&gt;=L122,"Ok","Aumentar h1 para "&amp;ROUNDUP(L120,0)&amp;" cm"))</f>
+        <v/>
+      </c>
+      <c r="O122" s="3" t="inlineStr">
+        <is>
+          <t>NBR 9062: h1 ≥ metade de H,cab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="K123" s="1" t="inlineStr">
+        <is>
           <t>A,cab</t>
         </is>
       </c>
-      <c r="L122" s="6">
-        <f>L37*L39+(L37+L32)/2*L119</f>
-        <v/>
-      </c>
-      <c r="M122" s="2" t="inlineStr">
+      <c r="L123" s="6">
+        <f>L37*L39+(L37+L32)/2*L120</f>
+        <v/>
+      </c>
+      <c r="M123" s="2" t="inlineStr">
         <is>
           <t>cm²</t>
         </is>
       </c>
-      <c r="O122" s="3" t="inlineStr">
+      <c r="O123" s="3" t="inlineStr">
         <is>
           <t>Área da cabeça vista de frente (retângulo + trapézio).</t>
         </is>
       </c>
     </row>
-    <row r="123">
-      <c r="K123" s="12" t="inlineStr">
+    <row r="124">
+      <c r="K124" s="12" t="inlineStr">
         <is>
           <t>4.2 Carga no balanço e classificação</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="K124" s="1" t="inlineStr">
-        <is>
-          <t>x,ap</t>
-        </is>
-      </c>
-      <c r="L124" s="6">
-        <f>MAX(0,MIN(L65,L43/2))</f>
-        <v/>
-      </c>
-      <c r="M124" s="2" t="inlineStr">
-        <is>
-          <t>cm</t>
-        </is>
-      </c>
-      <c r="O124" s="3" t="inlineStr">
-        <is>
-          <t>Parte do aparelho fora da face do pilar, de cada lado (item 1.7; limitada a a0/2).</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="K125" s="1" t="inlineStr">
         <is>
-          <t>Fd,c</t>
+          <t>x,ap</t>
         </is>
       </c>
       <c r="L125" s="6">
-        <f>L50*L124/L43</f>
+        <f>MAX(0,MIN(L66,L43/2))</f>
         <v/>
       </c>
       <c r="M125" s="2" t="inlineStr">
         <is>
-          <t>kN</t>
+          <t>cm</t>
         </is>
       </c>
       <c r="O125" s="3" t="inlineStr">
         <is>
-          <t>Carga de cálculo em cada balanço (pressão uniforme no apoio).</t>
+          <t>Parte do aparelho fora da face do pilar, de cada lado (item 1.7; limitada a a0/2).</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="K126" s="1" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>Fd,c</t>
         </is>
       </c>
       <c r="L126" s="6">
-        <f>L124/2</f>
+        <f>L51*L125/L43</f>
         <v/>
       </c>
       <c r="M126" s="2" t="inlineStr">
         <is>
-          <t>cm</t>
+          <t>kN</t>
         </is>
       </c>
       <c r="O126" s="3" t="inlineStr">
         <is>
-          <t>Distância da carga Fd,c até a face do pilar.</t>
+          <t>Carga de cálculo em cada balanço (pressão uniforme no apoio).</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="K127" s="1" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>a</t>
         </is>
       </c>
       <c r="L127" s="6">
-        <f>L120-L35-L107/20</f>
+        <f>L125/2</f>
         <v/>
       </c>
       <c r="M127" s="2" t="inlineStr">
@@ -3909,108 +3908,108 @@
       </c>
       <c r="O127" s="3" t="inlineStr">
         <is>
-          <t>Altura útil do consolo (até o eixo do tirante).</t>
+          <t>Distância da carga Fd,c até a face do pilar.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="K128" s="1" t="inlineStr">
         <is>
-          <t>a/d</t>
-        </is>
-      </c>
-      <c r="L128" s="22">
-        <f>IFERROR(L126/L127,0)</f>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="L128" s="6">
+        <f>L121-L35-L108/20</f>
         <v/>
       </c>
       <c r="M128" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>cm</t>
         </is>
       </c>
       <c r="O128" s="3" t="inlineStr">
         <is>
-          <t>Define o tipo de consolo.</t>
+          <t>Altura útil do consolo (até o eixo do tirante).</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="K129" s="1" t="inlineStr">
         <is>
+          <t>a/d</t>
+        </is>
+      </c>
+      <c r="L129" s="22">
+        <f>IFERROR(L127/L128,0)</f>
+        <v/>
+      </c>
+      <c r="M129" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O129" s="3" t="inlineStr">
+        <is>
+          <t>Define o tipo de consolo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="K130" s="1" t="inlineStr">
+        <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="L129" s="18">
-        <f>IF(L68&lt;&gt;"Consolo","Não se aplica (bloco)",IF(L124=0,"Balanço sem carga",IF(L128&lt;=0.5,"Muito curto",IF(L128&lt;=1,"Curto","Viga em balanço"))))</f>
-        <v/>
-      </c>
-      <c r="M129" s="2" t="inlineStr">
+      <c r="L130" s="18">
+        <f>IF(L69&lt;&gt;"Consolo","Não se aplica (bloco)",IF(L125=0,"Balanço sem carga",IF(L129&lt;=0.5,"Muito curto",IF(L129&lt;=1,"Curto","Viga em balanço"))))</f>
+        <v/>
+      </c>
+      <c r="M130" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="O129" s="3" t="inlineStr">
+      <c r="O130" s="3" t="inlineStr">
         <is>
           <t>a/d ≤ 0,5 muito curto | ≤ 1 curto | &gt; 1 viga em balanço.</t>
         </is>
       </c>
     </row>
-    <row r="130">
-      <c r="K130" s="12" t="inlineStr">
+    <row r="131">
+      <c r="K131" s="12" t="inlineStr">
         <is>
           <t>4.3 Armaduras do consolo</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="K131" s="1" t="inlineStr">
-        <is>
-          <t>μ,c</t>
-        </is>
-      </c>
-      <c r="L131" s="4" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="M131" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O131" s="3" t="inlineStr">
-        <is>
-          <t>Atrito do consolo muito curto (1,4 = monolítico).</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="K132" s="1" t="inlineStr">
         <is>
-          <t>As,m.curto</t>
-        </is>
-      </c>
-      <c r="L132" s="6">
-        <f>0.8*L125/(L131*L29)+L55/L29</f>
-        <v/>
+          <t>μ,c</t>
+        </is>
+      </c>
+      <c r="L132" s="4" t="n">
+        <v>1.4</v>
       </c>
       <c r="M132" s="2" t="inlineStr">
         <is>
-          <t>cm²</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O132" s="3" t="inlineStr">
         <is>
-          <t>Muito curto: 0,8·Fd/(μ·fyd) + Hd/fyd.</t>
+          <t>Atrito do consolo muito curto (1,4 = monolítico).</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="K133" s="1" t="inlineStr">
         <is>
-          <t>As,curto</t>
+          <t>As,m.curto</t>
         </is>
       </c>
       <c r="L133" s="6">
-        <f>(0.1+L128)*L125/L29+L55/L29</f>
+        <f>0.8*L126/(L132*L29)+L56/L29</f>
         <v/>
       </c>
       <c r="M133" s="2" t="inlineStr">
@@ -4020,18 +4019,18 @@
       </c>
       <c r="O133" s="3" t="inlineStr">
         <is>
-          <t>Curto: (0,1 + a/d)·Fd/fyd + Hd/fyd.</t>
+          <t>Muito curto: 0,8·Fd/(μ·fyd) + Hd/fyd.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="K134" s="1" t="inlineStr">
         <is>
-          <t>As,viga</t>
+          <t>As,curto</t>
         </is>
       </c>
       <c r="L134" s="6">
-        <f>IFERROR(L125*L126/(0.9*L127*L29),0)+L55/L29</f>
+        <f>(0.1+L129)*L126/L29+L56/L29</f>
         <v/>
       </c>
       <c r="M134" s="2" t="inlineStr">
@@ -4041,18 +4040,18 @@
       </c>
       <c r="O134" s="3" t="inlineStr">
         <is>
-          <t>Viga em balanço: Md/(0,9·d·fyd) + Hd/fyd, com Md = Fd·a.</t>
+          <t>Curto: (0,1 + a/d)·Fd/fyd + Hd/fyd.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="K135" s="1" t="inlineStr">
         <is>
-          <t>As,tir,c</t>
+          <t>As,viga</t>
         </is>
       </c>
       <c r="L135" s="6">
-        <f>IF(L124=0,0,IF(L128&lt;=0.5,L132,IF(L128&lt;=1,L133,L134)))</f>
+        <f>IFERROR(L126*L127/(0.9*L128*L29),0)+L56/L29</f>
         <v/>
       </c>
       <c r="M135" s="2" t="inlineStr">
@@ -4062,18 +4061,18 @@
       </c>
       <c r="O135" s="3" t="inlineStr">
         <is>
-          <t>Tirante do consolo: só a fórmula do tipo (vai ao item 3.1).</t>
+          <t>Viga em balanço: Md/(0,9·d·fyd) + Hd/fyd, com Md = Fd·a.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="K136" s="1" t="inlineStr">
         <is>
-          <t>As,mín</t>
+          <t>As,tir,c</t>
         </is>
       </c>
       <c r="L136" s="6">
-        <f>0.04*L27/(L29*10)*L33*L127</f>
+        <f>IF(L125=0,0,IF(L129&lt;=0.5,L133,IF(L129&lt;=1,L134,L135)))</f>
         <v/>
       </c>
       <c r="M136" s="2" t="inlineStr">
@@ -4083,174 +4082,174 @@
       </c>
       <c r="O136" s="3" t="inlineStr">
         <is>
-          <t>Armadura mínima do tirante: 0,04·(fcd/fyd)·b·d.</t>
+          <t>Tirante do consolo: só a fórmula do tipo (vai ao item 3.1).</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="K137" s="1" t="inlineStr">
         <is>
-          <t>k,cost</t>
+          <t>As,mín</t>
         </is>
       </c>
       <c r="L137" s="6">
-        <f>IF(L128&lt;=0.5,0.5,0.4)</f>
+        <f>0.04*L27/(L29*10)*L33*L128</f>
         <v/>
       </c>
       <c r="M137" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>cm²</t>
         </is>
       </c>
       <c r="O137" s="3" t="inlineStr">
         <is>
-          <t>Fração do tirante para a costura (0,5 muito curto; 0,4 curto).</t>
+          <t>Armadura mínima do tirante: 0,04·(fcd/fyd)·b·d.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="K138" s="1" t="inlineStr">
         <is>
-          <t>As,cost</t>
+          <t>k,cost</t>
         </is>
       </c>
       <c r="L138" s="6">
-        <f>IF(OR(L68&lt;&gt;"Consolo",L124&lt;=0,L128&gt;1),0,L137*L135)</f>
+        <f>IF(L129&lt;=0.5,0.5,0.4)</f>
         <v/>
       </c>
       <c r="M138" s="2" t="inlineStr">
         <is>
-          <t>cm²</t>
+          <t>-</t>
         </is>
       </c>
       <c r="O138" s="3" t="inlineStr">
         <is>
-          <t>Estribos horizontais em 2/3·d (só modelo Consolo; não se aplica a viga).</t>
+          <t>Fração do tirante para a costura (0,5 muito curto; 0,4 curto).</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="K139" s="1" t="inlineStr">
         <is>
-          <t>Ø</t>
-        </is>
-      </c>
-      <c r="L139" s="4" t="n">
-        <v>8</v>
+          <t>As,cost</t>
+        </is>
+      </c>
+      <c r="L139" s="6">
+        <f>IF(OR(L69&lt;&gt;"Consolo",L125&lt;=0,L129&gt;1),0,L138*L136)</f>
+        <v/>
       </c>
       <c r="M139" s="2" t="inlineStr">
         <is>
-          <t>mm</t>
+          <t>cm²</t>
         </is>
       </c>
       <c r="O139" s="3" t="inlineStr">
         <is>
-          <t>Bitola escolhida para a costura.</t>
+          <t>Estribos horizontais em 2/3·d (só modelo Consolo; não se aplica a viga).</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="K140" s="1" t="inlineStr">
         <is>
-          <t>ramos</t>
+          <t>Ø</t>
         </is>
       </c>
       <c r="L140" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="M140" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="O140" s="3" t="inlineStr">
         <is>
-          <t>Ramos de cada estribo de costura (estribo fechado = 2).</t>
+          <t>Bitola escolhida para a costura.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="K141" s="1" t="inlineStr">
         <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="L141" s="7">
-        <f>IF(L68&lt;&gt;"Consolo",0,MAX(2,ROUNDUP(L138/(L140*PI()*(L139/10)^2/4),0)))</f>
-        <v/>
+          <t>ramos</t>
+        </is>
+      </c>
+      <c r="L141" s="4" t="n">
+        <v>2</v>
       </c>
       <c r="M141" s="2" t="inlineStr">
         <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="N141" s="5">
-        <f>IF(L68&lt;&gt;"Consolo","Não se aplica (bloco)",IF(L128&gt;1,"Viga: estribos por cisalhamento","Ok"))</f>
-        <v/>
+          <t>-</t>
+        </is>
       </c>
       <c r="O141" s="3" t="inlineStr">
         <is>
-          <t>Quantidade de estribos de costura (mínimo 2; zero no modelo Bloco).</t>
+          <t>Ramos de cada estribo de costura (estribo fechado = 2).</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="K142" s="1" t="inlineStr">
         <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="L142" s="7">
+        <f>IF(L69&lt;&gt;"Consolo",0,MAX(2,ROUNDUP(L139/(L141*PI()*(L140/10)^2/4),0)))</f>
+        <v/>
+      </c>
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="N142" s="5">
+        <f>IF(L69&lt;&gt;"Consolo","Não se aplica (bloco)",IF(L129&gt;1,"Viga: estribos por cisalhamento","Ok"))</f>
+        <v/>
+      </c>
+      <c r="O142" s="3" t="inlineStr">
+        <is>
+          <t>Quantidade de estribos de costura (mínimo 2; zero no modelo Bloco).</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="K143" s="1" t="inlineStr">
+        <is>
           <t>s</t>
         </is>
       </c>
-      <c r="L142" s="7">
-        <f>IF(L141=0,0,ROUNDDOWN((2/3*L127)/L141,0))</f>
-        <v/>
-      </c>
-      <c r="M142" s="2" t="inlineStr">
+      <c r="L143" s="7">
+        <f>IF(L142=0,0,ROUNDDOWN((2/3*L128)/L142,0))</f>
+        <v/>
+      </c>
+      <c r="M143" s="2" t="inlineStr">
         <is>
           <t>cm</t>
         </is>
       </c>
-      <c r="O142" s="3" t="inlineStr">
+      <c r="O143" s="3" t="inlineStr">
         <is>
           <t>Espaçamento da costura, distribuída em 2/3·d abaixo do tirante.</t>
         </is>
       </c>
     </row>
-    <row r="143">
-      <c r="K143" s="12" t="inlineStr">
+    <row r="144">
+      <c r="K144" s="12" t="inlineStr">
         <is>
           <t>4.4 Biela (esmagamento do concreto)</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="K144" s="1" t="inlineStr">
-        <is>
-          <t>τwd</t>
-        </is>
-      </c>
-      <c r="L144" s="6">
-        <f>IFERROR(L125/(L33*L127)*10,0)</f>
-        <v/>
-      </c>
-      <c r="M144" s="2" t="inlineStr">
-        <is>
-          <t>MPa</t>
-        </is>
-      </c>
-      <c r="O144" s="3" t="inlineStr">
-        <is>
-          <t>Tensão de cisalhamento no consolo: Fd,c/(b·d).</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="K145" s="1" t="inlineStr">
         <is>
-          <t>τwu</t>
+          <t>τwd</t>
         </is>
       </c>
       <c r="L145" s="6">
-        <f>0.27*(1-L26/250)*L27</f>
+        <f>IFERROR(L126/(L33*L128)*10,0)</f>
         <v/>
       </c>
       <c r="M145" s="2" t="inlineStr">
@@ -4258,152 +4257,152 @@
           <t>MPa</t>
         </is>
       </c>
-      <c r="N145" s="5">
-        <f>IF(L68&lt;&gt;"Consolo","Não se aplica (bloco)",IF(L144&lt;=L145,"Ok","Aumentar H,cab ou b"))</f>
-        <v/>
-      </c>
       <c r="O145" s="3" t="inlineStr">
         <is>
-          <t>Limite: 0,27·(1 − fck/250)·fcd.</t>
+          <t>Tensão de cisalhamento no consolo: Fd,c/(b·d).</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="K146" s="1" t="inlineStr">
         <is>
+          <t>τwu</t>
+        </is>
+      </c>
+      <c r="L146" s="6">
+        <f>0.27*(1-L26/250)*L27</f>
+        <v/>
+      </c>
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="N146" s="5">
+        <f>IF(L69&lt;&gt;"Consolo","Não se aplica (bloco)",IF(L145&lt;=L146,"Ok","Aumentar H,cab ou b"))</f>
+        <v/>
+      </c>
+      <c r="O146" s="3" t="inlineStr">
+        <is>
+          <t>Limite: 0,27·(1 − fck/250)·fcd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="K147" s="1" t="inlineStr">
+        <is>
           <t>σ,pilar</t>
         </is>
       </c>
-      <c r="L146" s="6">
-        <f>L50/(L32*L33)*10</f>
-        <v/>
-      </c>
-      <c r="M146" s="2" t="inlineStr">
+      <c r="L147" s="6">
+        <f>L51/(L32*L33)*10</f>
+        <v/>
+      </c>
+      <c r="M147" s="2" t="inlineStr">
         <is>
           <t>MPa</t>
         </is>
       </c>
-      <c r="N146" s="5">
-        <f>IF(L146&lt;=0.85*L27,"Ok","Verificar pilar")</f>
-        <v/>
-      </c>
-      <c r="O146" s="3" t="inlineStr">
+      <c r="N147" s="5">
+        <f>IF(L147&lt;=0.85*L27,"Ok","Verificar pilar")</f>
+        <v/>
+      </c>
+      <c r="O147" s="3" t="inlineStr">
         <is>
           <t>Tensão média no fuste logo abaixo da cabeça.</t>
         </is>
       </c>
     </row>
-    <row r="147"/>
-    <row r="148">
-      <c r="K148" s="16" t="inlineStr">
+    <row r="148"/>
+    <row r="149">
+      <c r="K149" s="16" t="inlineStr">
         <is>
           <t>5 . APARELHO DE APOIO</t>
         </is>
       </c>
-      <c r="L148" s="19" t="n"/>
-      <c r="M148" s="19" t="n"/>
-      <c r="N148" s="19" t="n"/>
-      <c r="O148" s="19" t="n"/>
-      <c r="P148" s="19" t="n"/>
-      <c r="Q148" s="19" t="n"/>
-      <c r="R148" s="19" t="n"/>
-      <c r="S148" s="19" t="n"/>
-      <c r="T148" s="20" t="n"/>
-    </row>
-    <row r="149"/>
-    <row r="150">
-      <c r="K150" s="1" t="inlineStr">
-        <is>
-          <t>A,ap</t>
-        </is>
-      </c>
-      <c r="L150" s="22">
-        <f>(L43*L44-PI()*(L46/2)^2)/100^2</f>
-        <v/>
-      </c>
-      <c r="M150" s="2" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="O150" s="3" t="inlineStr">
-        <is>
-          <t>Área do aparelho descontado o furo.</t>
-        </is>
-      </c>
-    </row>
+      <c r="L149" s="19" t="n"/>
+      <c r="M149" s="19" t="n"/>
+      <c r="N149" s="19" t="n"/>
+      <c r="O149" s="19" t="n"/>
+      <c r="P149" s="19" t="n"/>
+      <c r="Q149" s="19" t="n"/>
+      <c r="R149" s="19" t="n"/>
+      <c r="S149" s="19" t="n"/>
+      <c r="T149" s="20" t="n"/>
+    </row>
+    <row r="150"/>
     <row r="151" s="15">
       <c r="K151" s="1" t="inlineStr">
         <is>
+          <t>A,ap</t>
+        </is>
+      </c>
+      <c r="L151" s="22">
+        <f>(L43*L44-2*L47*PI()*(L46/2)^2)/100^2</f>
+        <v/>
+      </c>
+      <c r="M151" s="2" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="O151" s="3" t="inlineStr">
+        <is>
+          <t>Área dos 2 aparelhos descontados todos os furos (2 × n,furos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="K152" s="1" t="inlineStr">
+        <is>
           <t>σ,ap</t>
         </is>
       </c>
-      <c r="L151" s="6">
-        <f>L50/L150/1000</f>
-        <v/>
-      </c>
-      <c r="M151" s="2" t="inlineStr">
+      <c r="L152" s="6">
+        <f>L51/L151/1000</f>
+        <v/>
+      </c>
+      <c r="M152" s="2" t="inlineStr">
         <is>
           <t>MPa</t>
         </is>
       </c>
-      <c r="N151" s="5">
-        <f>IF(L151&lt;=L47,"Ok","Aumentar apoio")</f>
-        <v/>
-      </c>
-      <c r="O151" s="3" t="inlineStr">
+      <c r="N152" s="5">
+        <f>IF(L152&lt;=L48,"Ok","Aumentar apoio")</f>
+        <v/>
+      </c>
+      <c r="O152" s="3" t="inlineStr">
         <is>
           <t>Tensão atuante no aparelho (Nd/A,ap).</t>
         </is>
       </c>
     </row>
-    <row r="152"/>
-    <row r="153">
-      <c r="K153" s="16" t="inlineStr">
+    <row r="153"/>
+    <row r="154">
+      <c r="K154" s="16" t="inlineStr">
         <is>
           <t>6 . PESO DE AÇO E TAXA</t>
         </is>
       </c>
-      <c r="L153" s="19" t="n"/>
-      <c r="M153" s="19" t="n"/>
-      <c r="N153" s="19" t="n"/>
-      <c r="O153" s="19" t="n"/>
-      <c r="P153" s="19" t="n"/>
-      <c r="Q153" s="19" t="n"/>
-      <c r="R153" s="19" t="n"/>
-      <c r="S153" s="19" t="n"/>
-      <c r="T153" s="20" t="n"/>
-    </row>
-    <row r="154"/>
-    <row r="155">
-      <c r="K155" s="1" t="inlineStr">
-        <is>
-          <t>Cintas</t>
-        </is>
-      </c>
-      <c r="L155" s="6">
-        <f>L96*PI()*(L94/10)^2/4*(2*(L37+L33)-8*L35+12)/100*L30</f>
-        <v/>
-      </c>
-      <c r="M155" s="2" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="O155" s="3" t="inlineStr">
-        <is>
-          <t>Cintas de fendilhamento (perímetro na cabeça + ganchos).</t>
-        </is>
-      </c>
-    </row>
+      <c r="L154" s="19" t="n"/>
+      <c r="M154" s="19" t="n"/>
+      <c r="N154" s="19" t="n"/>
+      <c r="O154" s="19" t="n"/>
+      <c r="P154" s="19" t="n"/>
+      <c r="Q154" s="19" t="n"/>
+      <c r="R154" s="19" t="n"/>
+      <c r="S154" s="19" t="n"/>
+      <c r="T154" s="20" t="n"/>
+    </row>
+    <row r="155"/>
     <row r="156">
       <c r="K156" s="1" t="inlineStr">
         <is>
-          <t>Tirante</t>
+          <t>Cintas</t>
         </is>
       </c>
       <c r="L156" s="6">
-        <f>L108*PI()*(L107/10)^2/4*(L37-2*L35+2*10*L107/10)/100*L30</f>
+        <f>L97*PI()*(L95/10)^2/4*(2*(L37+L33)-8*L35+12)/100*L30</f>
         <v/>
       </c>
       <c r="M156" s="2" t="inlineStr">
@@ -4413,18 +4412,18 @@
       </c>
       <c r="O156" s="3" t="inlineStr">
         <is>
-          <t>Tirante do topo (comprimento a,cab − 2c + 2 dobras de 10Ø).</t>
+          <t>Cintas de fendilhamento (perímetro na cabeça + ganchos).</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="K157" s="1" t="inlineStr">
         <is>
-          <t>Parede</t>
+          <t>Tirante</t>
         </is>
       </c>
       <c r="L157" s="6">
-        <f>L112*PI()*(L111/10)^2/4*(L37-2*L35+2*10*L111/10)/100*L30</f>
+        <f>L109*PI()*(L108/10)^2/4*(L37-2*L35+2*10*L108/10)/100*L30</f>
         <v/>
       </c>
       <c r="M157" s="2" t="inlineStr">
@@ -4434,18 +4433,18 @@
       </c>
       <c r="O157" s="3" t="inlineStr">
         <is>
-          <t>Parede oposta (mesmo critério de comprimento).</t>
+          <t>Tirante do topo (comprimento a,cab − 2c + 2 dobras de 10Ø).</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="K158" s="1" t="inlineStr">
         <is>
-          <t>Costura</t>
+          <t>Parede</t>
         </is>
       </c>
       <c r="L158" s="6">
-        <f>L141*PI()*(L139/10)^2/4*(2*(L37+L33)-8*L35+12)/100*L30</f>
+        <f>L113*PI()*(L112/10)^2/4*(L37-2*L35+2*10*L112/10)/100*L30</f>
         <v/>
       </c>
       <c r="M158" s="2" t="inlineStr">
@@ -4455,18 +4454,18 @@
       </c>
       <c r="O158" s="3" t="inlineStr">
         <is>
-          <t>Estribos de costura (perímetro na cabeça + ganchos).</t>
+          <t>Parede oposta (mesmo critério de comprimento).</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="K159" s="1" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Costura</t>
         </is>
       </c>
       <c r="L159" s="6">
-        <f>L155+L156+L157+L158</f>
+        <f>L142*PI()*(L140/10)^2/4*(2*(L37+L33)-8*L35+12)/100*L30</f>
         <v/>
       </c>
       <c r="M159" s="2" t="inlineStr">
@@ -4476,78 +4475,98 @@
       </c>
       <c r="O159" s="3" t="inlineStr">
         <is>
-          <t>Peso de aço destas armaduras.</t>
+          <t>Estribos de costura (perímetro na cabeça + ganchos).</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="K160" s="1" t="inlineStr">
         <is>
-          <t>Volume</t>
-        </is>
-      </c>
-      <c r="L160" s="22">
-        <f>(L32*L33*(L34-L120)+L122*L33)/100^3</f>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="L160" s="6">
+        <f>L156+L157+L158+L159</f>
         <v/>
       </c>
       <c r="M160" s="2" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="O160" s="3" t="inlineStr">
         <is>
-          <t>Volume de concreto: pilar (h,pil × b) + cabeça com mísulas.</t>
+          <t>Peso de aço destas armaduras.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="K161" s="1" t="inlineStr">
         <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="L161" s="22">
+        <f>(L32*L33*(L34-L121)+L123*L33)/100^3</f>
+        <v/>
+      </c>
+      <c r="M161" s="2" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="O161" s="3" t="inlineStr">
+        <is>
+          <t>Volume de concreto: pilar (h,pil × b) + cabeça com mísulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="K162" s="1" t="inlineStr">
+        <is>
           <t>Taxa</t>
         </is>
       </c>
-      <c r="L161" s="6">
-        <f>L159/L160</f>
-        <v/>
-      </c>
-      <c r="M161" s="2" t="inlineStr">
+      <c r="L162" s="6">
+        <f>L160/L161</f>
+        <v/>
+      </c>
+      <c r="M162" s="2" t="inlineStr">
         <is>
           <t>kg/m³</t>
         </is>
       </c>
-      <c r="O161" s="3" t="inlineStr">
+      <c r="O162" s="3" t="inlineStr">
         <is>
           <t>Taxa destas armaduras (sem a armadura do pilar).</t>
         </is>
       </c>
     </row>
-    <row r="162"/>
-    <row r="163">
-      <c r="K163" s="16" t="inlineStr">
+    <row r="163"/>
+    <row r="164">
+      <c r="K164" s="16" t="inlineStr">
         <is>
           <t>7 . DESENHO DA CABEÇA COM AS ARMADURAS CALCULADAS (atualiza automaticamente)</t>
         </is>
       </c>
-      <c r="L163" s="19" t="n"/>
-      <c r="M163" s="19" t="n"/>
-      <c r="N163" s="19" t="n"/>
-      <c r="O163" s="19" t="n"/>
-      <c r="P163" s="19" t="n"/>
-      <c r="Q163" s="19" t="n"/>
-      <c r="R163" s="19" t="n"/>
-      <c r="S163" s="19" t="n"/>
-      <c r="T163" s="20" t="n"/>
-    </row>
-    <row r="164"/>
-    <row r="165" ht="32.1" customHeight="1" s="15">
-      <c r="K165" s="14" t="inlineStr">
+      <c r="L164" s="19" t="n"/>
+      <c r="M164" s="19" t="n"/>
+      <c r="N164" s="19" t="n"/>
+      <c r="O164" s="19" t="n"/>
+      <c r="P164" s="19" t="n"/>
+      <c r="Q164" s="19" t="n"/>
+      <c r="R164" s="19" t="n"/>
+      <c r="S164" s="19" t="n"/>
+      <c r="T164" s="20" t="n"/>
+    </row>
+    <row r="165"/>
+    <row r="166" ht="32.1" customHeight="1" s="15">
+      <c r="K166" s="14" t="inlineStr">
         <is>
           <t>Gráfico de linhas (dispersão) desenhado a partir da tabela de coordenadas abaixo. Origem no topo da cabeça, no eixo do pilar; y negativo para baixo. Para detalhar outras armaduras no futuro, basta acrescentar um bloco de coordenadas e uma nova série no gráfico.</t>
         </is>
       </c>
     </row>
-    <row r="166"/>
     <row r="167"/>
     <row r="168"/>
     <row r="169"/>
@@ -4591,65 +4610,56 @@
     <row r="207"/>
     <row r="208"/>
     <row r="209"/>
-    <row r="210">
-      <c r="K210" s="17" t="inlineStr">
+    <row r="210"/>
+    <row r="211">
+      <c r="K211" s="17" t="inlineStr">
         <is>
           <t>Elemento</t>
         </is>
       </c>
-      <c r="L210" s="17" t="inlineStr">
+      <c r="L211" s="17" t="inlineStr">
         <is>
           <t>x (cm)</t>
         </is>
       </c>
-      <c r="M210" s="17" t="inlineStr">
+      <c r="M211" s="17" t="inlineStr">
         <is>
           <t>y (cm)</t>
         </is>
       </c>
-      <c r="N210" s="17" t="n"/>
-      <c r="O210" s="17" t="inlineStr">
+      <c r="N211" s="17" t="n"/>
+      <c r="O211" s="17" t="inlineStr">
         <is>
           <t>Observação</t>
         </is>
       </c>
     </row>
-    <row r="211">
-      <c r="K211" s="1" t="inlineStr">
+    <row r="212">
+      <c r="K212" s="1" t="inlineStr">
         <is>
           <t>Contorno</t>
         </is>
       </c>
-      <c r="L211" s="6">
-        <f>L32/2</f>
-        <v/>
-      </c>
-      <c r="M211" s="6">
-        <f>-(L120+MAX(40,L93-L120+10))</f>
-        <v/>
-      </c>
-      <c r="O211" s="3">
-        <f>"Contorno da cabeça e do pilar"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="212">
       <c r="L212" s="6">
         <f>L32/2</f>
         <v/>
       </c>
       <c r="M212" s="6">
-        <f>-L120</f>
+        <f>-(L121+MAX(40,L94-L121+10))</f>
+        <v/>
+      </c>
+      <c r="O212" s="3">
+        <f>"Contorno da cabeça e do pilar"</f>
         <v/>
       </c>
     </row>
     <row r="213">
       <c r="L213" s="6">
-        <f>L37/2</f>
+        <f>L32/2</f>
         <v/>
       </c>
       <c r="M213" s="6">
-        <f>-L39</f>
+        <f>-L121</f>
         <v/>
       </c>
     </row>
@@ -4659,13 +4669,13 @@
         <v/>
       </c>
       <c r="M214" s="6">
-        <f>0</f>
+        <f>-L39</f>
         <v/>
       </c>
     </row>
     <row r="215">
       <c r="L215" s="6">
-        <f>-L37/2</f>
+        <f>L37/2</f>
         <v/>
       </c>
       <c r="M215" s="6">
@@ -4679,17 +4689,17 @@
         <v/>
       </c>
       <c r="M216" s="6">
-        <f>-L39</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
     <row r="217">
       <c r="L217" s="6">
-        <f>-L32/2</f>
+        <f>-L37/2</f>
         <v/>
       </c>
       <c r="M217" s="6">
-        <f>-L120</f>
+        <f>-L39</f>
         <v/>
       </c>
     </row>
@@ -4699,36 +4709,36 @@
         <v/>
       </c>
       <c r="M218" s="6">
-        <f>-(L120+MAX(40,L93-L120+10))</f>
+        <f>-L121</f>
         <v/>
       </c>
     </row>
     <row r="219">
-      <c r="K219" s="1" t="inlineStr">
+      <c r="L219" s="6">
+        <f>-L32/2</f>
+        <v/>
+      </c>
+      <c r="M219" s="6">
+        <f>-(L121+MAX(40,L94-L121+10))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="220">
+      <c r="K220" s="1" t="inlineStr">
         <is>
           <t>Aparelho</t>
         </is>
       </c>
-      <c r="L219" s="6">
+      <c r="L220" s="6">
         <f>-(L37/2-L42)</f>
-        <v/>
-      </c>
-      <c r="M219" s="6">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="O219" s="3">
-        <f>"Aparelhos 2 × "&amp;L43/2&amp;" × "&amp;L44&amp;" cm (junta "&amp;2*(L37/2-L42-L43/2)&amp;" cm)"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="220">
-      <c r="L220" s="6">
-        <f>-(L37/2-L42-L43/2)</f>
         <v/>
       </c>
       <c r="M220" s="6">
         <f>0</f>
+        <v/>
+      </c>
+      <c r="O220" s="3">
+        <f>"Aparelhos 2 × "&amp;L43/2&amp;" × "&amp;L44&amp;" cm (junta "&amp;2*(L37/2-L42-L43/2)&amp;" cm)"</f>
         <v/>
       </c>
     </row>
@@ -4738,13 +4748,13 @@
         <v/>
       </c>
       <c r="M221" s="6">
-        <f>MAX(L45,2)</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
     <row r="222">
       <c r="L222" s="6">
-        <f>-(L37/2-L42)</f>
+        <f>-(L37/2-L42-L43/2)</f>
         <v/>
       </c>
       <c r="M222" s="6">
@@ -4758,27 +4768,27 @@
         <v/>
       </c>
       <c r="M223" s="6">
+        <f>MAX(L45,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="224">
+      <c r="L224" s="6">
+        <f>-(L37/2-L42)</f>
+        <v/>
+      </c>
+      <c r="M224" s="6">
         <f>0</f>
         <v/>
       </c>
     </row>
-    <row r="224">
-      <c r="L224" s="6" t="n"/>
-      <c r="M224" s="6" t="n"/>
-    </row>
     <row r="225">
-      <c r="L225" s="6">
-        <f>(L37/2-L42-L43/2)</f>
-        <v/>
-      </c>
-      <c r="M225" s="6">
-        <f>0</f>
-        <v/>
-      </c>
+      <c r="L225" s="6" t="n"/>
+      <c r="M225" s="6" t="n"/>
     </row>
     <row r="226">
       <c r="L226" s="6">
-        <f>L37/2-L42</f>
+        <f>(L37/2-L42-L43/2)</f>
         <v/>
       </c>
       <c r="M226" s="6">
@@ -4792,13 +4802,13 @@
         <v/>
       </c>
       <c r="M227" s="6">
-        <f>MAX(L45,2)</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
     <row r="228">
       <c r="L228" s="6">
-        <f>(L37/2-L42-L43/2)</f>
+        <f>L37/2-L42</f>
         <v/>
       </c>
       <c r="M228" s="6">
@@ -4812,46 +4822,46 @@
         <v/>
       </c>
       <c r="M229" s="6">
+        <f>MAX(L45,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="230">
+      <c r="L230" s="6">
+        <f>(L37/2-L42-L43/2)</f>
+        <v/>
+      </c>
+      <c r="M230" s="6">
         <f>0</f>
         <v/>
       </c>
     </row>
-    <row r="230">
-      <c r="K230" s="1" t="inlineStr">
+    <row r="231">
+      <c r="K231" s="1" t="inlineStr">
         <is>
           <t>Tirante</t>
         </is>
       </c>
-      <c r="L230" s="6">
-        <f>-(L37/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M230" s="6">
-        <f>(-(L35+L107/20))-(L107)</f>
-        <v/>
-      </c>
-      <c r="O230" s="3">
-        <f>"Tirante "&amp;L108&amp;" Ø"&amp;L107&amp;IF(L68="Bloco"," (bloco)"," (consolo)")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="231">
       <c r="L231" s="6">
         <f>-(L37/2-L35)</f>
         <v/>
       </c>
       <c r="M231" s="6">
-        <f>(-(L35+L107/20))</f>
+        <f>(-(L35+L108/20))-(L108)</f>
+        <v/>
+      </c>
+      <c r="O231" s="3">
+        <f>"Tirante "&amp;L109&amp;" Ø"&amp;L108&amp;IF(L69="Bloco"," (bloco)"," (consolo)")</f>
         <v/>
       </c>
     </row>
     <row r="232">
       <c r="L232" s="6">
-        <f>(L37/2-L35)</f>
+        <f>-(L37/2-L35)</f>
         <v/>
       </c>
       <c r="M232" s="6">
-        <f>(-(L35+L107/20))</f>
+        <f>(-(L35+L108/20))</f>
         <v/>
       </c>
     </row>
@@ -4861,707 +4871,717 @@
         <v/>
       </c>
       <c r="M233" s="6">
-        <f>(-(L35+L107/20))-(L107)</f>
+        <f>(-(L35+L108/20))</f>
         <v/>
       </c>
     </row>
     <row r="234">
-      <c r="K234" s="1" t="inlineStr">
+      <c r="L234" s="6">
+        <f>(L37/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M234" s="6">
+        <f>(-(L35+L108/20))-(L108)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="235">
+      <c r="K235" s="1" t="inlineStr">
         <is>
           <t>Costura</t>
         </is>
       </c>
-      <c r="L234" s="6">
-        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
-        <v/>
-      </c>
-      <c r="M234" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))</f>
-        <v/>
-      </c>
-      <c r="O234" s="3">
-        <f>IF(L141=0,"Costura – não se aplica (bloco)","Costura "&amp;L141&amp;" Ø"&amp;L139&amp;" c/"&amp;L142)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="235">
       <c r="L235" s="6">
-        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L142=0,L325,-(IF((-((-(L35+L108/20))-IF(1&lt;=L142,1,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(1&lt;=L142,1,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(1&lt;=L142,1,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M235" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(1&lt;=L141,1,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="236"/>
-    <row r="237">
-      <c r="L237" s="6">
-        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
-        <v/>
-      </c>
-      <c r="M237" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(1&lt;=L142,1,1)*L143))</f>
+        <v/>
+      </c>
+      <c r="O235" s="3">
+        <f>IF(L142=0,"Costura – não se aplica (bloco)","Costura "&amp;L142&amp;" Ø"&amp;L140&amp;" c/"&amp;L143)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="236">
+      <c r="L236" s="6">
+        <f>IF(L142=0,L325,(IF((-((-(L35+L108/20))-IF(1&lt;=L142,1,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(1&lt;=L142,1,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(1&lt;=L142,1,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
+        <v/>
+      </c>
+      <c r="M236" s="6">
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(1&lt;=L142,1,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="237"/>
     <row r="238">
       <c r="L238" s="6">
-        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L142=0,L325,-(IF((-((-(L35+L108/20))-IF(2&lt;=L142,2,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(2&lt;=L142,2,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(2&lt;=L142,2,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M238" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(2&lt;=L141,2,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="239"/>
-    <row r="240">
-      <c r="L240" s="6">
-        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
-        <v/>
-      </c>
-      <c r="M240" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(2&lt;=L142,2,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="239">
+      <c r="L239" s="6">
+        <f>IF(L142=0,L325,(IF((-((-(L35+L108/20))-IF(2&lt;=L142,2,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(2&lt;=L142,2,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(2&lt;=L142,2,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
+        <v/>
+      </c>
+      <c r="M239" s="6">
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(2&lt;=L142,2,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="240"/>
     <row r="241">
       <c r="L241" s="6">
-        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L142=0,L325,-(IF((-((-(L35+L108/20))-IF(3&lt;=L142,3,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(3&lt;=L142,3,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(3&lt;=L142,3,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M241" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(3&lt;=L141,3,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="242"/>
-    <row r="243">
-      <c r="L243" s="6">
-        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
-        <v/>
-      </c>
-      <c r="M243" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(3&lt;=L142,3,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="242">
+      <c r="L242" s="6">
+        <f>IF(L142=0,L325,(IF((-((-(L35+L108/20))-IF(3&lt;=L142,3,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(3&lt;=L142,3,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(3&lt;=L142,3,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
+        <v/>
+      </c>
+      <c r="M242" s="6">
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(3&lt;=L142,3,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="243"/>
     <row r="244">
       <c r="L244" s="6">
-        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L142=0,L325,-(IF((-((-(L35+L108/20))-IF(4&lt;=L142,4,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(4&lt;=L142,4,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(4&lt;=L142,4,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M244" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(4&lt;=L141,4,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="245"/>
-    <row r="246">
-      <c r="L246" s="6">
-        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
-        <v/>
-      </c>
-      <c r="M246" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(4&lt;=L142,4,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="245">
+      <c r="L245" s="6">
+        <f>IF(L142=0,L325,(IF((-((-(L35+L108/20))-IF(4&lt;=L142,4,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(4&lt;=L142,4,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(4&lt;=L142,4,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
+        <v/>
+      </c>
+      <c r="M245" s="6">
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(4&lt;=L142,4,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="246"/>
     <row r="247">
       <c r="L247" s="6">
-        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L142=0,L325,-(IF((-((-(L35+L108/20))-IF(5&lt;=L142,5,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(5&lt;=L142,5,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(5&lt;=L142,5,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M247" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(5&lt;=L141,5,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="248"/>
-    <row r="249">
-      <c r="L249" s="6">
-        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
-        <v/>
-      </c>
-      <c r="M249" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(5&lt;=L142,5,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="248">
+      <c r="L248" s="6">
+        <f>IF(L142=0,L325,(IF((-((-(L35+L108/20))-IF(5&lt;=L142,5,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(5&lt;=L142,5,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(5&lt;=L142,5,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
+        <v/>
+      </c>
+      <c r="M248" s="6">
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(5&lt;=L142,5,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="249"/>
     <row r="250">
       <c r="L250" s="6">
-        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L142=0,L325,-(IF((-((-(L35+L108/20))-IF(6&lt;=L142,6,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(6&lt;=L142,6,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(6&lt;=L142,6,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M250" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(6&lt;=L141,6,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="251"/>
-    <row r="252">
-      <c r="L252" s="6">
-        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
-        <v/>
-      </c>
-      <c r="M252" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(6&lt;=L142,6,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="251">
+      <c r="L251" s="6">
+        <f>IF(L142=0,L325,(IF((-((-(L35+L108/20))-IF(6&lt;=L142,6,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(6&lt;=L142,6,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(6&lt;=L142,6,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
+        <v/>
+      </c>
+      <c r="M251" s="6">
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(6&lt;=L142,6,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="252"/>
     <row r="253">
       <c r="L253" s="6">
-        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L142=0,L325,-(IF((-((-(L35+L108/20))-IF(7&lt;=L142,7,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(7&lt;=L142,7,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(7&lt;=L142,7,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M253" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(7&lt;=L141,7,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="254"/>
-    <row r="255">
-      <c r="L255" s="6">
-        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
-        <v/>
-      </c>
-      <c r="M255" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(7&lt;=L142,7,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="254">
+      <c r="L254" s="6">
+        <f>IF(L142=0,L325,(IF((-((-(L35+L108/20))-IF(7&lt;=L142,7,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(7&lt;=L142,7,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(7&lt;=L142,7,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
+        <v/>
+      </c>
+      <c r="M254" s="6">
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(7&lt;=L142,7,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="255"/>
     <row r="256">
       <c r="L256" s="6">
-        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L142=0,L325,-(IF((-((-(L35+L108/20))-IF(8&lt;=L142,8,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(8&lt;=L142,8,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(8&lt;=L142,8,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M256" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(8&lt;=L141,8,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="257"/>
-    <row r="258">
-      <c r="L258" s="6">
-        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
-        <v/>
-      </c>
-      <c r="M258" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(8&lt;=L142,8,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="257">
+      <c r="L257" s="6">
+        <f>IF(L142=0,L325,(IF((-((-(L35+L108/20))-IF(8&lt;=L142,8,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(8&lt;=L142,8,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(8&lt;=L142,8,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
+        <v/>
+      </c>
+      <c r="M257" s="6">
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(8&lt;=L142,8,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="258"/>
     <row r="259">
       <c r="L259" s="6">
-        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L142=0,L325,-(IF((-((-(L35+L108/20))-IF(9&lt;=L142,9,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(9&lt;=L142,9,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(9&lt;=L142,9,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M259" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(9&lt;=L141,9,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="260"/>
-    <row r="261">
-      <c r="L261" s="6">
-        <f>IF(L141=0,L324,-(IF((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
-        <v/>
-      </c>
-      <c r="M261" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(9&lt;=L142,9,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="260">
+      <c r="L260" s="6">
+        <f>IF(L142=0,L325,(IF((-((-(L35+L108/20))-IF(9&lt;=L142,9,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(9&lt;=L142,9,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(9&lt;=L142,9,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
+        <v/>
+      </c>
+      <c r="M260" s="6">
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(9&lt;=L142,9,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="261"/>
     <row r="262">
       <c r="L262" s="6">
-        <f>IF(L141=0,L324,(IF((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))&lt;=L39,L37,IF((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))&lt;=L120,L37-2*((-((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))-L39)*L118/MAX(L119,0.001),L32))/2-L35))</f>
+        <f>IF(L142=0,L325,-(IF((-((-(L35+L108/20))-IF(10&lt;=L142,10,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(10&lt;=L142,10,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(10&lt;=L142,10,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
         <v/>
       </c>
       <c r="M262" s="6">
-        <f>IF(L141=0,M324,((-(L35+L107/20))-IF(10&lt;=L141,10,1)*L142))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="263"/>
-    <row r="264">
-      <c r="K264" s="1" t="inlineStr">
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(10&lt;=L142,10,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="263">
+      <c r="L263" s="6">
+        <f>IF(L142=0,L325,(IF((-((-(L35+L108/20))-IF(10&lt;=L142,10,1)*L143))&lt;=L39,L37,IF((-((-(L35+L108/20))-IF(10&lt;=L142,10,1)*L143))&lt;=L121,L37-2*((-((-(L35+L108/20))-IF(10&lt;=L142,10,1)*L143))-L39)*L119/MAX(L120,0.001),L32))/2-L35))</f>
+        <v/>
+      </c>
+      <c r="M263" s="6">
+        <f>IF(L142=0,M325,((-(L35+L108/20))-IF(10&lt;=L142,10,1)*L143))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="264"/>
+    <row r="265">
+      <c r="K265" s="1" t="inlineStr">
         <is>
           <t>Cintas</t>
         </is>
       </c>
-      <c r="L264" s="6">
-        <f>-(IF((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M264" s="6">
-        <f>(-(IF(1&lt;=L96,1,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-      <c r="O264" s="3">
-        <f>"Cintas "&amp;L96&amp;" Ø"&amp;L94&amp;" c/"&amp;L97</f>
-        <v/>
-      </c>
-    </row>
-    <row r="265">
       <c r="L265" s="6">
-        <f>(IF((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(1&lt;=L96,1,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(1&lt;=L97,1,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(1&lt;=L97,1,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(1&lt;=L97,1,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M265" s="6">
-        <f>(-(IF(1&lt;=L96,1,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="266"/>
-    <row r="267">
-      <c r="L267" s="6">
-        <f>-(IF((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M267" s="6">
-        <f>(-(IF(2&lt;=L96,2,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
+        <f>(-(IF(1&lt;=L97,1,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+      <c r="O265" s="3">
+        <f>"Cintas "&amp;L97&amp;" Ø"&amp;L95&amp;" c/"&amp;L98</f>
+        <v/>
+      </c>
+    </row>
+    <row r="266">
+      <c r="L266" s="6">
+        <f>(IF((-(-(IF(1&lt;=L97,1,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(1&lt;=L97,1,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(1&lt;=L97,1,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M266" s="6">
+        <f>(-(IF(1&lt;=L97,1,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="267"/>
     <row r="268">
       <c r="L268" s="6">
-        <f>(IF((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(2&lt;=L96,2,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(2&lt;=L97,2,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(2&lt;=L97,2,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(2&lt;=L97,2,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M268" s="6">
-        <f>(-(IF(2&lt;=L96,2,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="269"/>
-    <row r="270">
-      <c r="L270" s="6">
-        <f>-(IF((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M270" s="6">
-        <f>(-(IF(3&lt;=L96,3,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
+        <f>(-(IF(2&lt;=L97,2,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="269">
+      <c r="L269" s="6">
+        <f>(IF((-(-(IF(2&lt;=L97,2,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(2&lt;=L97,2,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(2&lt;=L97,2,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M269" s="6">
+        <f>(-(IF(2&lt;=L97,2,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="270"/>
     <row r="271">
       <c r="L271" s="6">
-        <f>(IF((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(3&lt;=L96,3,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(3&lt;=L97,3,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(3&lt;=L97,3,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(3&lt;=L97,3,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M271" s="6">
-        <f>(-(IF(3&lt;=L96,3,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="272"/>
-    <row r="273">
-      <c r="L273" s="6">
-        <f>-(IF((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M273" s="6">
-        <f>(-(IF(4&lt;=L96,4,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
+        <f>(-(IF(3&lt;=L97,3,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="272">
+      <c r="L272" s="6">
+        <f>(IF((-(-(IF(3&lt;=L97,3,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(3&lt;=L97,3,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(3&lt;=L97,3,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M272" s="6">
+        <f>(-(IF(3&lt;=L97,3,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="273"/>
     <row r="274">
       <c r="L274" s="6">
-        <f>(IF((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(4&lt;=L96,4,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(4&lt;=L97,4,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(4&lt;=L97,4,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(4&lt;=L97,4,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M274" s="6">
-        <f>(-(IF(4&lt;=L96,4,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="275"/>
-    <row r="276">
-      <c r="L276" s="6">
-        <f>-(IF((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M276" s="6">
-        <f>(-(IF(5&lt;=L96,5,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
+        <f>(-(IF(4&lt;=L97,4,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="275">
+      <c r="L275" s="6">
+        <f>(IF((-(-(IF(4&lt;=L97,4,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(4&lt;=L97,4,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(4&lt;=L97,4,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M275" s="6">
+        <f>(-(IF(4&lt;=L97,4,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="276"/>
     <row r="277">
       <c r="L277" s="6">
-        <f>(IF((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(5&lt;=L96,5,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(5&lt;=L97,5,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(5&lt;=L97,5,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(5&lt;=L97,5,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M277" s="6">
-        <f>(-(IF(5&lt;=L96,5,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="278"/>
-    <row r="279">
-      <c r="L279" s="6">
-        <f>-(IF((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M279" s="6">
-        <f>(-(IF(6&lt;=L96,6,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
+        <f>(-(IF(5&lt;=L97,5,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="278">
+      <c r="L278" s="6">
+        <f>(IF((-(-(IF(5&lt;=L97,5,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(5&lt;=L97,5,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(5&lt;=L97,5,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M278" s="6">
+        <f>(-(IF(5&lt;=L97,5,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="279"/>
     <row r="280">
       <c r="L280" s="6">
-        <f>(IF((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(6&lt;=L96,6,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(6&lt;=L97,6,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(6&lt;=L97,6,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(6&lt;=L97,6,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M280" s="6">
-        <f>(-(IF(6&lt;=L96,6,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="281"/>
-    <row r="282">
-      <c r="L282" s="6">
-        <f>-(IF((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M282" s="6">
-        <f>(-(IF(7&lt;=L96,7,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
+        <f>(-(IF(6&lt;=L97,6,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="281">
+      <c r="L281" s="6">
+        <f>(IF((-(-(IF(6&lt;=L97,6,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(6&lt;=L97,6,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(6&lt;=L97,6,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M281" s="6">
+        <f>(-(IF(6&lt;=L97,6,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="282"/>
     <row r="283">
       <c r="L283" s="6">
-        <f>(IF((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(7&lt;=L96,7,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(7&lt;=L97,7,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(7&lt;=L97,7,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(7&lt;=L97,7,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M283" s="6">
-        <f>(-(IF(7&lt;=L96,7,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="284"/>
-    <row r="285">
-      <c r="L285" s="6">
-        <f>-(IF((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M285" s="6">
-        <f>(-(IF(8&lt;=L96,8,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
+        <f>(-(IF(7&lt;=L97,7,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="284">
+      <c r="L284" s="6">
+        <f>(IF((-(-(IF(7&lt;=L97,7,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(7&lt;=L97,7,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(7&lt;=L97,7,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M284" s="6">
+        <f>(-(IF(7&lt;=L97,7,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="285"/>
     <row r="286">
       <c r="L286" s="6">
-        <f>(IF((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(8&lt;=L96,8,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(8&lt;=L97,8,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(8&lt;=L97,8,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(8&lt;=L97,8,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M286" s="6">
-        <f>(-(IF(8&lt;=L96,8,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="287"/>
-    <row r="288">
-      <c r="L288" s="6">
-        <f>-(IF((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M288" s="6">
-        <f>(-(IF(9&lt;=L96,9,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
+        <f>(-(IF(8&lt;=L97,8,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="287">
+      <c r="L287" s="6">
+        <f>(IF((-(-(IF(8&lt;=L97,8,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(8&lt;=L97,8,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(8&lt;=L97,8,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M287" s="6">
+        <f>(-(IF(8&lt;=L97,8,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="288"/>
     <row r="289">
       <c r="L289" s="6">
-        <f>(IF((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(9&lt;=L96,9,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(9&lt;=L97,9,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(9&lt;=L97,9,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(9&lt;=L97,9,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M289" s="6">
-        <f>(-(IF(9&lt;=L96,9,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="290"/>
-    <row r="291">
-      <c r="L291" s="6">
-        <f>-(IF((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M291" s="6">
-        <f>(-(IF(10&lt;=L96,10,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
+        <f>(-(IF(9&lt;=L97,9,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="290">
+      <c r="L290" s="6">
+        <f>(IF((-(-(IF(9&lt;=L97,9,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(9&lt;=L97,9,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(9&lt;=L97,9,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M290" s="6">
+        <f>(-(IF(9&lt;=L97,9,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="291"/>
     <row r="292">
       <c r="L292" s="6">
-        <f>(IF((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(10&lt;=L96,10,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(10&lt;=L97,10,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(10&lt;=L97,10,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(10&lt;=L97,10,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M292" s="6">
-        <f>(-(IF(10&lt;=L96,10,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="293"/>
-    <row r="294">
-      <c r="L294" s="6">
-        <f>-(IF((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M294" s="6">
-        <f>(-(IF(11&lt;=L96,11,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
+        <f>(-(IF(10&lt;=L97,10,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="293">
+      <c r="L293" s="6">
+        <f>(IF((-(-(IF(10&lt;=L97,10,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(10&lt;=L97,10,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(10&lt;=L97,10,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M293" s="6">
+        <f>(-(IF(10&lt;=L97,10,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="294"/>
     <row r="295">
       <c r="L295" s="6">
-        <f>(IF((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(11&lt;=L96,11,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(11&lt;=L97,11,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(11&lt;=L97,11,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(11&lt;=L97,11,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M295" s="6">
-        <f>(-(IF(11&lt;=L96,11,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="296"/>
-    <row r="297">
-      <c r="L297" s="6">
-        <f>-(IF((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M297" s="6">
-        <f>(-(IF(12&lt;=L96,12,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
+        <f>(-(IF(11&lt;=L97,11,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="296">
+      <c r="L296" s="6">
+        <f>(IF((-(-(IF(11&lt;=L97,11,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(11&lt;=L97,11,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(11&lt;=L97,11,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M296" s="6">
+        <f>(-(IF(11&lt;=L97,11,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="297"/>
     <row r="298">
       <c r="L298" s="6">
-        <f>(IF((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(12&lt;=L96,12,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(12&lt;=L97,12,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(12&lt;=L97,12,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(12&lt;=L97,12,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M298" s="6">
-        <f>(-(IF(12&lt;=L96,12,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="299"/>
-    <row r="300">
-      <c r="L300" s="6">
-        <f>-(IF((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M300" s="6">
-        <f>(-(IF(13&lt;=L96,13,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
+        <f>(-(IF(12&lt;=L97,12,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="299">
+      <c r="L299" s="6">
+        <f>(IF((-(-(IF(12&lt;=L97,12,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(12&lt;=L97,12,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(12&lt;=L97,12,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M299" s="6">
+        <f>(-(IF(12&lt;=L97,12,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="300"/>
     <row r="301">
       <c r="L301" s="6">
-        <f>(IF((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(13&lt;=L96,13,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(13&lt;=L97,13,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(13&lt;=L97,13,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(13&lt;=L97,13,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M301" s="6">
-        <f>(-(IF(13&lt;=L96,13,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="302"/>
-    <row r="303">
-      <c r="L303" s="6">
-        <f>-(IF((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M303" s="6">
-        <f>(-(IF(14&lt;=L96,14,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
+        <f>(-(IF(13&lt;=L97,13,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="302">
+      <c r="L302" s="6">
+        <f>(IF((-(-(IF(13&lt;=L97,13,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(13&lt;=L97,13,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(13&lt;=L97,13,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M302" s="6">
+        <f>(-(IF(13&lt;=L97,13,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="303"/>
     <row r="304">
       <c r="L304" s="6">
-        <f>(IF((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(14&lt;=L96,14,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(14&lt;=L97,14,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(14&lt;=L97,14,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(14&lt;=L97,14,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M304" s="6">
-        <f>(-(IF(14&lt;=L96,14,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="305"/>
-    <row r="306">
-      <c r="L306" s="6">
-        <f>-(IF((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M306" s="6">
-        <f>(-(IF(15&lt;=L96,15,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
+        <f>(-(IF(14&lt;=L97,14,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="305">
+      <c r="L305" s="6">
+        <f>(IF((-(-(IF(14&lt;=L97,14,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(14&lt;=L97,14,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(14&lt;=L97,14,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M305" s="6">
+        <f>(-(IF(14&lt;=L97,14,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="306"/>
     <row r="307">
       <c r="L307" s="6">
-        <f>(IF((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(15&lt;=L96,15,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(15&lt;=L97,15,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(15&lt;=L97,15,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(15&lt;=L97,15,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M307" s="6">
-        <f>(-(IF(15&lt;=L96,15,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="309">
-      <c r="L309" s="6">
-        <f>-(IF((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M309" s="6">
-        <f>(-(IF(16&lt;=L96,16,1)-0.5)*L97)</f>
+        <f>(-(IF(15&lt;=L97,15,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="308">
+      <c r="L308" s="6">
+        <f>(IF((-(-(IF(15&lt;=L97,15,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(15&lt;=L97,15,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(15&lt;=L97,15,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M308" s="6">
+        <f>(-(IF(15&lt;=L97,15,1)-0.5)*L98)</f>
         <v/>
       </c>
     </row>
     <row r="310">
       <c r="L310" s="6">
-        <f>(IF((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(16&lt;=L96,16,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(16&lt;=L97,16,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(16&lt;=L97,16,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(16&lt;=L97,16,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M310" s="6">
-        <f>(-(IF(16&lt;=L96,16,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="312">
-      <c r="L312" s="6">
-        <f>-(IF((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M312" s="6">
-        <f>(-(IF(17&lt;=L96,17,1)-0.5)*L97)</f>
+        <f>(-(IF(16&lt;=L97,16,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="311">
+      <c r="L311" s="6">
+        <f>(IF((-(-(IF(16&lt;=L97,16,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(16&lt;=L97,16,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(16&lt;=L97,16,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M311" s="6">
+        <f>(-(IF(16&lt;=L97,16,1)-0.5)*L98)</f>
         <v/>
       </c>
     </row>
     <row r="313">
       <c r="L313" s="6">
-        <f>(IF((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(17&lt;=L96,17,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(17&lt;=L97,17,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(17&lt;=L97,17,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(17&lt;=L97,17,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M313" s="6">
-        <f>(-(IF(17&lt;=L96,17,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="315">
-      <c r="L315" s="6">
-        <f>-(IF((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M315" s="6">
-        <f>(-(IF(18&lt;=L96,18,1)-0.5)*L97)</f>
+        <f>(-(IF(17&lt;=L97,17,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="314">
+      <c r="L314" s="6">
+        <f>(IF((-(-(IF(17&lt;=L97,17,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(17&lt;=L97,17,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(17&lt;=L97,17,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M314" s="6">
+        <f>(-(IF(17&lt;=L97,17,1)-0.5)*L98)</f>
         <v/>
       </c>
     </row>
     <row r="316">
       <c r="L316" s="6">
-        <f>(IF((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(18&lt;=L96,18,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(18&lt;=L97,18,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(18&lt;=L97,18,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(18&lt;=L97,18,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M316" s="6">
-        <f>(-(IF(18&lt;=L96,18,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="318">
-      <c r="L318" s="6">
-        <f>-(IF((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M318" s="6">
-        <f>(-(IF(19&lt;=L96,19,1)-0.5)*L97)</f>
+        <f>(-(IF(18&lt;=L97,18,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="317">
+      <c r="L317" s="6">
+        <f>(IF((-(-(IF(18&lt;=L97,18,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(18&lt;=L97,18,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(18&lt;=L97,18,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M317" s="6">
+        <f>(-(IF(18&lt;=L97,18,1)-0.5)*L98)</f>
         <v/>
       </c>
     </row>
     <row r="319">
       <c r="L319" s="6">
-        <f>(IF((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(19&lt;=L96,19,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(19&lt;=L97,19,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(19&lt;=L97,19,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(19&lt;=L97,19,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M319" s="6">
-        <f>(-(IF(19&lt;=L96,19,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="321">
-      <c r="L321" s="6">
-        <f>-(IF((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
-        <v/>
-      </c>
-      <c r="M321" s="6">
-        <f>(-(IF(20&lt;=L96,20,1)-0.5)*L97)</f>
+        <f>(-(IF(19&lt;=L97,19,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="320">
+      <c r="L320" s="6">
+        <f>(IF((-(-(IF(19&lt;=L97,19,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(19&lt;=L97,19,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(19&lt;=L97,19,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M320" s="6">
+        <f>(-(IF(19&lt;=L97,19,1)-0.5)*L98)</f>
         <v/>
       </c>
     </row>
     <row r="322">
       <c r="L322" s="6">
-        <f>(IF((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))&lt;=L39,L37,IF((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))&lt;=L120,L37-2*((-(-(IF(20&lt;=L96,20,1)-0.5)*L97))-L39)*L118/MAX(L119,0.001),L32))/2-L35)</f>
+        <f>-(IF((-(-(IF(20&lt;=L97,20,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(20&lt;=L97,20,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(20&lt;=L97,20,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
         <v/>
       </c>
       <c r="M322" s="6">
-        <f>(-(IF(20&lt;=L96,20,1)-0.5)*L97)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="324">
-      <c r="K324" s="1" t="inlineStr">
+        <f>(-(IF(20&lt;=L97,20,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="323">
+      <c r="L323" s="6">
+        <f>(IF((-(-(IF(20&lt;=L97,20,1)-0.5)*L98))&lt;=L39,L37,IF((-(-(IF(20&lt;=L97,20,1)-0.5)*L98))&lt;=L121,L37-2*((-(-(IF(20&lt;=L97,20,1)-0.5)*L98))-L39)*L119/MAX(L120,0.001),L32))/2-L35)</f>
+        <v/>
+      </c>
+      <c r="M323" s="6">
+        <f>(-(IF(20&lt;=L97,20,1)-0.5)*L98)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="325">
+      <c r="K325" s="1" t="inlineStr">
         <is>
           <t>Eixo</t>
         </is>
       </c>
-      <c r="L324" s="6">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="M324" s="6">
-        <f>MAX(L45,2)+8</f>
-        <v/>
-      </c>
-      <c r="O324" s="3">
-        <f>"Eixo do pilar"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="325">
       <c r="L325" s="6">
         <f>0</f>
         <v/>
       </c>
       <c r="M325" s="6">
-        <f>-(L120+MAX(40,L93-L120+10))</f>
+        <f>MAX(L45,2)+8</f>
+        <v/>
+      </c>
+      <c r="O325" s="3">
+        <f>"Eixo do pilar"</f>
         <v/>
       </c>
     </row>
     <row r="326">
-      <c r="K326" s="1" t="inlineStr">
+      <c r="L326" s="6">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="M326" s="6">
+        <f>-(L121+MAX(40,L94-L121+10))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="327">
+      <c r="K327" s="1" t="inlineStr">
         <is>
           <t>Moldura</t>
         </is>
       </c>
-      <c r="L326" s="6">
-        <f>-MAX(L37+30,(L120+MAX(40,L93-L120+10))+25)/2</f>
-        <v/>
-      </c>
-      <c r="M326" s="6">
+      <c r="L327" s="6">
+        <f>-MAX(L37+30,(L121+MAX(40,L94-L121+10))+25)/2</f>
+        <v/>
+      </c>
+      <c r="M327" s="6">
         <f>15</f>
         <v/>
       </c>
-      <c r="O326" s="3">
+      <c r="O327" s="3">
         <f>"(moldura – mantém a escala)"</f>
         <v/>
       </c>
     </row>
-    <row r="327">
-      <c r="L327" s="6">
-        <f>MAX(L37+30,(L120+MAX(40,L93-L120+10))+25)/2</f>
-        <v/>
-      </c>
-      <c r="M327" s="6">
-        <f>15-MAX(L37+30,(L120+MAX(40,L93-L120+10))+25)</f>
+    <row r="328">
+      <c r="L328" s="6">
+        <f>MAX(L37+30,(L121+MAX(40,L94-L121+10))+25)/2</f>
+        <v/>
+      </c>
+      <c r="M328" s="6">
+        <f>15-MAX(L37+30,(L121+MAX(40,L94-L121+10))+25)</f>
         <v/>
       </c>
     </row>
@@ -5569,61 +5589,61 @@
   <mergeCells count="29">
     <mergeCell ref="L17:M17"/>
     <mergeCell ref="L7:M7"/>
+    <mergeCell ref="K70:T70"/>
     <mergeCell ref="L16:M16"/>
-    <mergeCell ref="K148:T148"/>
+    <mergeCell ref="K166:T166"/>
+    <mergeCell ref="K73:T73"/>
     <mergeCell ref="L8:T8"/>
-    <mergeCell ref="K116:T116"/>
     <mergeCell ref="L13:M13"/>
-    <mergeCell ref="K101:T101"/>
+    <mergeCell ref="K65:T65"/>
+    <mergeCell ref="K2:T2"/>
     <mergeCell ref="K19:T19"/>
     <mergeCell ref="L12:M12"/>
     <mergeCell ref="K4:T4"/>
-    <mergeCell ref="K69:T69"/>
     <mergeCell ref="L15:M15"/>
-    <mergeCell ref="K74:T74"/>
     <mergeCell ref="L14:M14"/>
-    <mergeCell ref="K114:T114"/>
+    <mergeCell ref="K164:T164"/>
+    <mergeCell ref="K154:T154"/>
     <mergeCell ref="L10:M10"/>
-    <mergeCell ref="K163:T163"/>
-    <mergeCell ref="K64:T64"/>
-    <mergeCell ref="K153:T153"/>
+    <mergeCell ref="K100:T100"/>
     <mergeCell ref="K1:T1"/>
     <mergeCell ref="L9:M9"/>
-    <mergeCell ref="K99:T99"/>
-    <mergeCell ref="K72:T72"/>
-    <mergeCell ref="K165:T165"/>
     <mergeCell ref="O6:T6"/>
     <mergeCell ref="L6:M6"/>
+    <mergeCell ref="K75:T75"/>
+    <mergeCell ref="K102:T102"/>
+    <mergeCell ref="K149:T149"/>
+    <mergeCell ref="K115:T115"/>
     <mergeCell ref="L11:M11"/>
-    <mergeCell ref="K2:T2"/>
+    <mergeCell ref="K117:T117"/>
   </mergeCells>
-  <conditionalFormatting sqref="N7:N8 N9:N17 N68 N79 N84 N96 N108 N112 N121 N141 N145:N146 N151">
+  <conditionalFormatting sqref="N7:N8 N9:N17 N69 N80 N85 N97 N109 N113 N122 N142 N146:N147 N152">
     <cfRule type="beginsWith" priority="1" operator="beginsWith" dxfId="0" text="Ok">
       <formula>LEFT(N7,2)="Ok"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N7:N8 N9:N17 N79 N84 N96 N108 N112 N121 N141 N145:N146 N151">
+  <conditionalFormatting sqref="N7:N8 N9:N17 N80 N85 N97 N109 N113 N122 N142 N146:N147 N152">
     <cfRule type="beginsWith" priority="2" operator="beginsWith" dxfId="1" text="Não se aplica">
       <formula>LEFT(N7,13)="Não se aplica"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="L51" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="L52" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Sim,Não"</formula1>
     </dataValidation>
-    <dataValidation sqref="L52" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>$O$57:$O$62</formula1>
+    <dataValidation sqref="L53" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>$O$58:$O$63</formula1>
     </dataValidation>
-    <dataValidation sqref="L67" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
+    <dataValidation sqref="L68" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
       <formula1>"Automático,Bloco,Consolo"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
   <pageSetup orientation="portrait" paperSize="9" scale="74" fitToHeight="0"/>
   <rowBreaks count="3" manualBreakCount="3">
-    <brk id="71" min="10" max="19" man="1"/>
-    <brk id="113" min="0" max="16383" man="1"/>
-    <brk id="162" min="0" max="16383" man="1"/>
+    <brk id="72" min="10" max="19" man="1"/>
+    <brk id="114" min="0" max="16383" man="1"/>
+    <brk id="163" min="0" max="16383" man="1"/>
   </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Tirante do topo: área pelo modelo adotado; parede oposta só no Bloco
No modelo Consolo o tirante vai de face a face com a área do consolo
(item 4.3); a parede oposta da referência passa a valer só no modelo Bloco.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q3cH5Ra5NbDLqkpmKm8CnH
</commit_message>
<xml_diff>
--- a/34 - Bloco Parcialmente carregado.xlsx
+++ b/34 - Bloco Parcialmente carregado.xlsx
@@ -1974,7 +1974,7 @@
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>Barras horizontais no topo (face carregada + consolo) – item 3.1</t>
+          <t>Tirante do topo, de face a face (área do consolo ou da referência) – item 3.1</t>
         </is>
       </c>
     </row>
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="L12" s="18">
-        <f>L113&amp;" Ø"&amp;L112</f>
+        <f>IF(L113=0,"Não se aplica (consolo)",L113&amp;" Ø"&amp;L112)</f>
         <v/>
       </c>
       <c r="M12" s="20" t="n"/>
@@ -2987,7 +2987,7 @@
     </row>
     <row r="70" ht="48" customHeight="1" s="15">
       <c r="K70" s="21">
-        <f>IF(L69="Bloco","⚠ BLOCO PARCIALMENTE CARREGADO – aparelho todo sobre o pilar. Armaduras: cintas de fendilhamento (item 2: direções h e b + regra 0,25·Nd da referência), tirante do topo pela referência (item 3.1) e parede oposta (3.2). O consolo (item 4) não se aplica: sem costura.",IF(L66&lt;=0,"⚠ CONSOLO forçado, mas o aparelho não passa da face do pilar: a mísula não recebe carga – use o modelo Bloco.","⚠ CONSOLO – o aparelho passa "&amp;ROUND(L66,1)&amp;" cm da face do pilar de cada lado: a mísula é um consolo "&amp;LOWER(L130)&amp;" (a/d = "&amp;ROUND(L129,2)&amp;"). Armaduras: tirante do topo e costura pelo consolo (item 4, NBR 9062); cintas de fendilhamento só na direção b (b0 → b), pois na direção h a carga converge para o pilar e não espalha (item 2). Parede oposta (3.2) mantida."))</f>
+        <f>IF(L69="Bloco","⚠ BLOCO PARCIALMENTE CARREGADO – aparelho todo sobre o pilar. Armaduras: cintas de fendilhamento (item 2: direções h e b + regra 0,25·Nd da referência), tirante do topo pela referência (item 3.1) e parede oposta (3.2). O consolo (item 4) não se aplica: sem costura.",IF(L66&lt;=0,"⚠ CONSOLO forçado, mas o aparelho não passa da face do pilar: a mísula não recebe carga – use o modelo Bloco.","⚠ CONSOLO – o aparelho passa "&amp;ROUND(L66,1)&amp;" cm da face do pilar de cada lado: a mísula é um consolo "&amp;LOWER(L130)&amp;" (a/d = "&amp;ROUND(L129,2)&amp;"). Armaduras: tirante do topo e costura pelo consolo (item 4, NBR 9062); cintas de fendilhamento só na direção b (b0 → b), pois na direção h a carga converge para o pilar e não espalha (item 2). Parede oposta (3.2) não se aplica: o tirante vai de face a face."))</f>
         <v/>
       </c>
     </row>
@@ -3471,7 +3471,7 @@
     <row r="100">
       <c r="K100" s="16" t="inlineStr">
         <is>
-          <t>3 . TIRANTES NO TOPO DA CABEÇA (planilha de referência)</t>
+          <t>3 . TIRANTE NO TOPO DA CABEÇA (detalhamento – área vem do modelo adotado)</t>
         </is>
       </c>
       <c r="L100" s="19" t="n"/>
@@ -3488,14 +3488,14 @@
     <row r="102" ht="32.1" customHeight="1" s="15">
       <c r="K102" s="14" t="inlineStr">
         <is>
-          <t>Barras horizontais logo abaixo do topo. Modelo BLOCO: tirante pela regra da referência (0,25·Nd + 1,8·Hd). Modelo CONSOLO: o tirante da face carregada é o tirante do consolo (item 4) – usa-se o maior entre o consolo e a armadura mínima.</t>
+          <t>Barras horizontais logo abaixo do topo, contínuas de uma face à outra da cabeça e ancoradas nas duas faces externas (dobras/laços). Modelo CONSOLO: a área é a do tirante do consolo (item 4.3), nunca menor que a mínima – a regra da referência (As,ref) NÃO é usada. Modelo BLOCO: área pela regra da referência (0,25·Nd + 1,8·Hd) e parede oposta (3.2).</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="K103" s="12" t="inlineStr">
         <is>
-          <t>3.1 Tirante da face carregada</t>
+          <t>3.1 Tirante do topo (contínuo, de face a face)</t>
         </is>
       </c>
     </row>
@@ -3516,7 +3516,7 @@
       </c>
       <c r="O104" s="3" t="inlineStr">
         <is>
-          <t>Referência: (0,25·Nd + 1,8·Hd)/fyd – modelo Bloco.</t>
+          <t>Referência: (0,25·Nd + 1,8·Hd)/fyd – só no modelo Bloco (no Consolo é só informativo).</t>
         </is>
       </c>
     </row>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="O105" s="3" t="inlineStr">
         <is>
-          <t>Tirante exigido pelo consolo (item 4.3) – modelo Consolo.</t>
+          <t>Tirante do consolo (item 4.3) – é esta a área no modelo Consolo.</t>
         </is>
       </c>
     </row>
@@ -3577,6 +3577,10 @@
           <t>cm²</t>
         </is>
       </c>
+      <c r="N107" s="5">
+        <f>IF(L69="Bloco","Ok – pela referência (bloco)","Ok – pelo consolo (item 4.3)")</f>
+        <v/>
+      </c>
       <c r="O107" s="3" t="inlineStr">
         <is>
           <t>Área do tirante: Bloco = As,ref; Consolo = maior entre As,cons e As,mín.</t>
@@ -3631,7 +3635,7 @@
     <row r="110">
       <c r="K110" s="12" t="inlineStr">
         <is>
-          <t>3.2 Parede oposta</t>
+          <t>3.2 Parede oposta (só modelo Bloco)</t>
         </is>
       </c>
     </row>
@@ -3683,7 +3687,7 @@
         </is>
       </c>
       <c r="L113" s="7">
-        <f>MAX(2,ROUNDUP(L111/(PI()*(L112/10)^2/4),0))</f>
+        <f>IF(L69&lt;&gt;"Bloco",0,MAX(2,ROUNDUP(L111/(PI()*(L112/10)^2/4),0)))</f>
         <v/>
       </c>
       <c r="M113" s="2" t="inlineStr">
@@ -3692,12 +3696,12 @@
         </is>
       </c>
       <c r="N113" s="5">
-        <f>"Ok"</f>
+        <f>IF(L69&lt;&gt;"Bloco","Não se aplica (consolo)","Ok")</f>
         <v/>
       </c>
       <c r="O113" s="3" t="inlineStr">
         <is>
-          <t>Quantidade de barras da parede oposta (mínimo 2).</t>
+          <t>Barras da parede oposta (mínimo 2). No Consolo o tirante já vai de face a face: não se aplica.</t>
         </is>
       </c>
     </row>
@@ -5617,12 +5621,12 @@
     <mergeCell ref="L11:M11"/>
     <mergeCell ref="K117:T117"/>
   </mergeCells>
-  <conditionalFormatting sqref="N7:N8 N9:N17 N69 N80 N85 N97 N109 N113 N122 N142 N146:N147 N152">
+  <conditionalFormatting sqref="N7:N8 N9:N17 N69 N80 N85 N97 N107 N109 N113 N122 N142 N146:N147 N152">
     <cfRule type="beginsWith" priority="1" operator="beginsWith" dxfId="0" text="Ok">
       <formula>LEFT(N7,2)="Ok"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N7:N8 N9:N17 N80 N85 N97 N109 N113 N122 N142 N146:N147 N152">
+  <conditionalFormatting sqref="N7:N8 N9:N17 N80 N85 N97 N107 N109 N113 N122 N142 N146:N147 N152">
     <cfRule type="beginsWith" priority="2" operator="beginsWith" dxfId="1" text="Não se aplica">
       <formula>LEFT(N7,13)="Não se aplica"</formula>
     </cfRule>

</xml_diff>